<commit_message>
Updates with cohort feedback on questions.
</commit_message>
<xml_diff>
--- a/longitudinal/data_processing_elements_longitudinal-MSN.xlsx
+++ b/longitudinal/data_processing_elements_longitudinal-MSN.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Computer\twey working files\ProPASS\MSN\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\twey\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{10079B67-3558-4762-AE1B-F0D7FC727299}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BC304EF5-0DB6-4985-9753-0050D9150C16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="1840" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MSN" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1704" uniqueCount="664">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1736" uniqueCount="671">
   <si>
     <t>index</t>
   </si>
@@ -2234,9 +2234,6 @@
     <t>PSQI_comp1_subjective_sleepquality</t>
   </si>
   <si>
-    <t>recode(1=0; 2=0; 3=1; 4=1; ELSE=NA)</t>
-  </si>
-  <si>
     <t>The study-specific variable categories 0 = Very good and 1 = Fairly good were coded as DataSchema variable category 0 = Never/Rarely. The study-specific variable categories  2 = Fairly bad and 3 = Very bad were coded as DataSchema variable category 1 = Some difficulties.</t>
   </si>
   <si>
@@ -2290,15 +2287,6 @@
 In a typical week during the past 4 weeks, did you do heavy exercise (such as aerobics, aquajogging, rope skipping, or heavy strenght training)?</t>
   </si>
   <si>
-    <t>Study-specific variables are about activities "in a typical week during the past 4 weeks". Activities included were: fast cycling, jogging, swimming, tennis, teamsport, and heavy exercise. Walking, slow cycling, and light exercise were not included.
-A positive response to any sport activity was coded as DataSchema category 1 = Yes. DataSchema category 0 = No could not be coded.</t>
-  </si>
-  <si>
-    <t>case_when(
-activity_Q04_done == 1 | activity_Q09_done ==1 | activity_Q10_done == 1 | activity_Q11_done ==1 | activity_Q12_done ==1 | activity_Q14_done == 1 ~ 1L ; 
-ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
     <t>Based on the variables in the online data dictionary. Are all variables available and part of the input dataset? Confirm if available in follow-up. If so, confirm variable names.</t>
   </si>
   <si>
@@ -2366,6 +2354,45 @@
     <t>case_when(
 !is.na(nit_alcoholtot.ph2) &amp; nit_alcoholtot.ph2 != -888 ~ as.numeric(nit_alcoholtot.ph2)*7 ; 
 ELSE ~ NA_real_)</t>
+  </si>
+  <si>
+    <t>Confirmed same format.</t>
+  </si>
+  <si>
+    <t>Not in follow-up, but could take from baseline. Changed to impossible, add comment.</t>
+  </si>
+  <si>
+    <t>Not available in follow-up, but available in baseline.</t>
+  </si>
+  <si>
+    <t>smoking_unitsperday.ph2 is available but needs to be requested.</t>
+  </si>
+  <si>
+    <t>Available, only at FUP, but need to request.
+recode(1=0; 2=0; 3=1; 4=1; ELSE=NA)</t>
+  </si>
+  <si>
+    <t>Available, but need to request.</t>
+  </si>
+  <si>
+    <t>Available, but need to request.
+case_when(
+activity_Q04_done == 1 | activity_Q09_done ==1 | activity_Q10_done == 1 | activity_Q11_done ==1 | activity_Q12_done ==1 | activity_Q14_done == 1 ~ 1L ; 
+ELSE ~ NA_integer_)
+Study-specific variables are about activities "in a typical week during the past 4 weeks". Activities included were: fast cycling, jogging, swimming, tennis, teamsport, and heavy exercise. Walking, slow cycling, and light exercise were not included.
+A positive response to any sport activity was coded as DataSchema category 1 = Yes. DataSchema category 0 = No could not be coded.</t>
+  </si>
+  <si>
+    <t>Available, need to request.</t>
+  </si>
+  <si>
+    <t>Available, but need to request and probably to clean. 
+To request and evaluate, but might not be compatible.</t>
+  </si>
+  <si>
+    <t>Available, but need to request and probably to clean. 
+To request and evaluate, but might not be compatible.
+Will be empty unless said yes to cancer other than skin cancer.</t>
   </si>
 </sst>
 </file>
@@ -2833,7 +2860,8 @@
     <col min="26" max="26" width="50.7109375" style="1" customWidth="1"/>
     <col min="27" max="27" width="61" style="1" customWidth="1"/>
     <col min="28" max="28" width="53" style="1" bestFit="1" customWidth="1"/>
-    <col min="29" max="16384" width="28.7109375" style="3"/>
+    <col min="29" max="29" width="43.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="30" max="16384" width="28.7109375" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:32" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3162,6 +3190,9 @@
       <c r="AA6" s="11" t="s">
         <v>608</v>
       </c>
+      <c r="AC6" s="3" t="s">
+        <v>661</v>
+      </c>
     </row>
     <row r="7" spans="1:32" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
@@ -3520,17 +3551,20 @@
       <c r="P14" s="3" t="s">
         <v>32</v>
       </c>
+      <c r="U14" s="3" t="s">
+        <v>663</v>
+      </c>
       <c r="V14" s="5" t="s">
-        <v>119</v>
+        <v>89</v>
       </c>
       <c r="W14" s="5" t="s">
-        <v>119</v>
+        <v>90</v>
       </c>
       <c r="X14" s="5" t="s">
-        <v>119</v>
+        <v>89</v>
       </c>
       <c r="Y14" s="5" t="s">
-        <v>119</v>
+        <v>89</v>
       </c>
       <c r="Z14" s="1" t="s">
         <v>118</v>
@@ -3540,6 +3574,9 @@
       </c>
       <c r="AB14" s="1" t="s">
         <v>612</v>
+      </c>
+      <c r="AC14" s="3" t="s">
+        <v>662</v>
       </c>
     </row>
     <row r="15" spans="1:32" ht="75" x14ac:dyDescent="0.25">
@@ -3954,7 +3991,7 @@
         <v>146</v>
       </c>
       <c r="M23" s="1" t="s">
-        <v>659</v>
+        <v>656</v>
       </c>
       <c r="N23" s="3" t="s">
         <v>174</v>
@@ -3975,7 +4012,7 @@
         <v>175</v>
       </c>
       <c r="AB23" s="1" t="s">
-        <v>660</v>
+        <v>657</v>
       </c>
     </row>
     <row r="24" spans="1:28" ht="60" x14ac:dyDescent="0.25">
@@ -4001,7 +4038,7 @@
         <v>152</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>659</v>
+        <v>656</v>
       </c>
       <c r="N24" s="3" t="s">
         <v>174</v>
@@ -4022,7 +4059,7 @@
         <v>178</v>
       </c>
       <c r="AB24" s="1" t="s">
-        <v>660</v>
+        <v>657</v>
       </c>
     </row>
     <row r="25" spans="1:28" ht="45" x14ac:dyDescent="0.25">
@@ -4618,7 +4655,7 @@
         <v>248</v>
       </c>
       <c r="AB37" s="1" t="s">
-        <v>661</v>
+        <v>658</v>
       </c>
     </row>
     <row r="38" spans="1:28" ht="45" x14ac:dyDescent="0.25">
@@ -5016,13 +5053,13 @@
         <v>103</v>
       </c>
       <c r="Y45" s="4" t="s">
-        <v>663</v>
+        <v>660</v>
       </c>
       <c r="Z45" s="1" t="s">
         <v>289</v>
       </c>
       <c r="AB45" s="1" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
     </row>
     <row r="46" spans="1:28" ht="60" x14ac:dyDescent="0.25">
@@ -5174,7 +5211,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="49" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:29" ht="45" x14ac:dyDescent="0.25">
       <c r="A49" s="3">
         <v>48</v>
       </c>
@@ -5213,17 +5250,17 @@
       <c r="P49" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="V49" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="W49" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="X49" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y49" s="8" t="s">
-        <v>89</v>
+      <c r="V49" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="W49" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="X49" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="Y49" s="5" t="s">
+        <v>119</v>
       </c>
       <c r="Z49" s="1" t="s">
         <v>311</v>
@@ -5234,8 +5271,11 @@
       <c r="AB49" s="1" t="s">
         <v>616</v>
       </c>
-    </row>
-    <row r="50" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC49" s="3" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="50" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A50" s="3">
         <v>49</v>
       </c>
@@ -5277,7 +5317,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="51" spans="1:28" ht="135" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:29" ht="135" x14ac:dyDescent="0.25">
       <c r="A51" s="3">
         <v>50</v>
       </c>
@@ -5339,7 +5379,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="52" spans="1:28" ht="75" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:29" ht="75" x14ac:dyDescent="0.25">
       <c r="A52" s="3">
         <v>51</v>
       </c>
@@ -5380,31 +5420,34 @@
         <v>626</v>
       </c>
       <c r="U52" s="3" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="V52" s="5" t="s">
-        <v>33</v>
+        <v>119</v>
       </c>
       <c r="W52" s="5" t="s">
-        <v>62</v>
+        <v>119</v>
       </c>
       <c r="X52" s="5" t="s">
-        <v>72</v>
+        <v>119</v>
       </c>
       <c r="Y52" s="5" t="s">
-        <v>628</v>
+        <v>119</v>
       </c>
       <c r="Z52" s="1" t="s">
         <v>325</v>
       </c>
       <c r="AA52" s="11" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="AB52" s="1" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="53" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+        <v>629</v>
+      </c>
+      <c r="AC52" s="1" t="s">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="53" spans="1:29" ht="45" x14ac:dyDescent="0.25">
       <c r="A53" s="3">
         <v>52</v>
       </c>
@@ -5452,7 +5495,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="54" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:29" ht="45" x14ac:dyDescent="0.25">
       <c r="A54" s="3">
         <v>53</v>
       </c>
@@ -5497,7 +5540,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="55" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:29" ht="45" x14ac:dyDescent="0.25">
       <c r="A55" s="3">
         <v>54</v>
       </c>
@@ -5542,7 +5585,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="56" spans="1:28" ht="315" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:29" ht="315" x14ac:dyDescent="0.25">
       <c r="A56" s="3">
         <v>55</v>
       </c>
@@ -5587,7 +5630,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="57" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:29" ht="45" x14ac:dyDescent="0.25">
       <c r="A57" s="3">
         <v>56</v>
       </c>
@@ -5635,7 +5678,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="58" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:29" ht="45" x14ac:dyDescent="0.25">
       <c r="A58" s="3">
         <v>57</v>
       </c>
@@ -5684,7 +5727,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="59" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:29" ht="45" x14ac:dyDescent="0.25">
       <c r="A59" s="3">
         <v>58</v>
       </c>
@@ -5733,7 +5776,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="60" spans="1:28" ht="135" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:29" ht="135" x14ac:dyDescent="0.25">
       <c r="A60" s="3">
         <v>59</v>
       </c>
@@ -5778,7 +5821,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="61" spans="1:28" ht="90" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:29" ht="90" x14ac:dyDescent="0.25">
       <c r="A61" s="3">
         <v>60</v>
       </c>
@@ -5807,14 +5850,14 @@
         <v>355</v>
       </c>
       <c r="N61" s="1" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="O61" s="11"/>
       <c r="P61" s="3" t="s">
         <v>32</v>
       </c>
       <c r="T61" s="3" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="V61" s="5" t="s">
         <v>119</v>
@@ -5832,13 +5875,16 @@
         <v>356</v>
       </c>
       <c r="AA61" s="11" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="AB61" s="1" t="s">
-        <v>634</v>
-      </c>
-    </row>
-    <row r="62" spans="1:28" ht="105" x14ac:dyDescent="0.25">
+        <v>633</v>
+      </c>
+      <c r="AC61" s="3" t="s">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="62" spans="1:29" ht="105" x14ac:dyDescent="0.25">
       <c r="A62" s="3">
         <v>61</v>
       </c>
@@ -5883,7 +5929,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="63" spans="1:28" ht="135" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:29" ht="255" x14ac:dyDescent="0.25">
       <c r="A63" s="3">
         <v>62</v>
       </c>
@@ -5912,10 +5958,10 @@
         <v>94</v>
       </c>
       <c r="M63" s="11" t="s">
+        <v>636</v>
+      </c>
+      <c r="N63" s="1" t="s">
         <v>637</v>
-      </c>
-      <c r="N63" s="1" t="s">
-        <v>638</v>
       </c>
       <c r="O63" s="1" t="s">
         <v>522</v>
@@ -5924,34 +5970,35 @@
         <v>32</v>
       </c>
       <c r="T63" s="3" t="s">
-        <v>639</v>
-      </c>
-      <c r="U63" s="11" t="s">
-        <v>640</v>
-      </c>
+        <v>638</v>
+      </c>
+      <c r="U63" s="11"/>
       <c r="V63" s="11" t="s">
-        <v>33</v>
+        <v>119</v>
       </c>
       <c r="W63" s="11" t="s">
-        <v>62</v>
+        <v>119</v>
       </c>
       <c r="X63" s="11" t="s">
-        <v>103</v>
+        <v>119</v>
       </c>
       <c r="Y63" s="11" t="s">
-        <v>641</v>
+        <v>119</v>
       </c>
       <c r="Z63" s="1" t="s">
         <v>365</v>
       </c>
       <c r="AA63" s="11" t="s">
-        <v>642</v>
+        <v>639</v>
       </c>
       <c r="AB63" s="1" t="s">
-        <v>635</v>
-      </c>
-    </row>
-    <row r="64" spans="1:28" ht="30" x14ac:dyDescent="0.25">
+        <v>634</v>
+      </c>
+      <c r="AC63" s="1" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="64" spans="1:29" ht="30" x14ac:dyDescent="0.25">
       <c r="A64" s="3">
         <v>63</v>
       </c>
@@ -5996,7 +6043,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="65" spans="1:27" ht="60" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:29" ht="60" x14ac:dyDescent="0.25">
       <c r="A65" s="3">
         <v>64</v>
       </c>
@@ -6047,7 +6094,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="66" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:29" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A66" s="3">
         <v>65</v>
       </c>
@@ -6098,7 +6145,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="67" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:29" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A67" s="3">
         <v>66</v>
       </c>
@@ -6149,7 +6196,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="68" spans="1:27" ht="75" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:29" ht="75" x14ac:dyDescent="0.25">
       <c r="A68" s="3">
         <v>67</v>
       </c>
@@ -6199,7 +6246,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="69" spans="1:27" ht="165" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:29" ht="165" x14ac:dyDescent="0.25">
       <c r="A69" s="3">
         <v>68</v>
       </c>
@@ -6255,7 +6302,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="70" spans="1:27" ht="75" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:29" ht="75" x14ac:dyDescent="0.25">
       <c r="A70" s="3">
         <v>69</v>
       </c>
@@ -6290,26 +6337,29 @@
       <c r="P70" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="V70" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="W70" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="X70" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y70" s="4" t="s">
-        <v>89</v>
+      <c r="V70" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="W70" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="X70" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="Y70" s="5" t="s">
+        <v>119</v>
       </c>
       <c r="Z70" s="1" t="s">
         <v>416</v>
       </c>
       <c r="AA70" s="11" t="s">
-        <v>643</v>
-      </c>
-    </row>
-    <row r="71" spans="1:27" ht="75" x14ac:dyDescent="0.25">
+        <v>640</v>
+      </c>
+      <c r="AC70" s="3" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="71" spans="1:29" ht="75" x14ac:dyDescent="0.25">
       <c r="A71" s="3">
         <v>70</v>
       </c>
@@ -6349,26 +6399,29 @@
       <c r="P71" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="V71" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="W71" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="X71" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y71" s="8" t="s">
-        <v>89</v>
+      <c r="V71" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="W71" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="X71" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="Y71" s="5" t="s">
+        <v>119</v>
       </c>
       <c r="Z71" s="1" t="s">
         <v>423</v>
       </c>
       <c r="AA71" s="11" t="s">
-        <v>643</v>
-      </c>
-    </row>
-    <row r="72" spans="1:27" ht="75" x14ac:dyDescent="0.25">
+        <v>640</v>
+      </c>
+      <c r="AC71" s="3" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="72" spans="1:29" ht="75" x14ac:dyDescent="0.25">
       <c r="A72" s="3">
         <v>71</v>
       </c>
@@ -6408,26 +6461,29 @@
       <c r="P72" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="V72" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="W72" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="X72" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y72" s="8" t="s">
-        <v>89</v>
+      <c r="V72" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="W72" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="X72" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="Y72" s="5" t="s">
+        <v>119</v>
       </c>
       <c r="Z72" s="1" t="s">
         <v>430</v>
       </c>
       <c r="AA72" s="11" t="s">
-        <v>643</v>
-      </c>
-    </row>
-    <row r="73" spans="1:27" ht="75" x14ac:dyDescent="0.25">
+        <v>640</v>
+      </c>
+      <c r="AC72" s="3" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="73" spans="1:29" ht="75" x14ac:dyDescent="0.25">
       <c r="A73" s="3">
         <v>72</v>
       </c>
@@ -6467,26 +6523,29 @@
       <c r="P73" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="V73" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="W73" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="X73" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y73" s="8" t="s">
-        <v>89</v>
+      <c r="V73" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="W73" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="X73" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="Y73" s="5" t="s">
+        <v>119</v>
       </c>
       <c r="Z73" s="1" t="s">
         <v>436</v>
       </c>
       <c r="AA73" s="11" t="s">
-        <v>643</v>
-      </c>
-    </row>
-    <row r="74" spans="1:27" ht="45" x14ac:dyDescent="0.25">
+        <v>640</v>
+      </c>
+      <c r="AC73" s="3" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="74" spans="1:29" ht="45" x14ac:dyDescent="0.25">
       <c r="A74" s="3">
         <v>73</v>
       </c>
@@ -6534,7 +6593,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="75" spans="1:27" ht="45" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:29" ht="45" x14ac:dyDescent="0.25">
       <c r="A75" s="3">
         <v>74</v>
       </c>
@@ -6582,7 +6641,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="76" spans="1:27" ht="45" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:29" ht="45" x14ac:dyDescent="0.25">
       <c r="A76" s="3">
         <v>75</v>
       </c>
@@ -6620,17 +6679,17 @@
       <c r="P76" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="V76" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="W76" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="X76" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y76" s="4" t="s">
-        <v>89</v>
+      <c r="V76" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="W76" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="X76" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="Y76" s="5" t="s">
+        <v>119</v>
       </c>
       <c r="Z76" s="1" t="s">
         <v>451</v>
@@ -6638,8 +6697,11 @@
       <c r="AA76" s="11" t="s">
         <v>615</v>
       </c>
-    </row>
-    <row r="77" spans="1:27" ht="45" x14ac:dyDescent="0.25">
+      <c r="AC76" s="3" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="77" spans="1:29" ht="45" x14ac:dyDescent="0.25">
       <c r="A77" s="3">
         <v>76</v>
       </c>
@@ -6679,17 +6741,17 @@
       <c r="P77" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="V77" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="W77" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="X77" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y77" s="4" t="s">
-        <v>89</v>
+      <c r="V77" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="W77" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="X77" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="Y77" s="5" t="s">
+        <v>119</v>
       </c>
       <c r="Z77" s="1" t="s">
         <v>458</v>
@@ -6697,8 +6759,11 @@
       <c r="AA77" s="11" t="s">
         <v>615</v>
       </c>
-    </row>
-    <row r="78" spans="1:27" ht="45" x14ac:dyDescent="0.25">
+      <c r="AC77" s="3" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="78" spans="1:29" ht="45" x14ac:dyDescent="0.25">
       <c r="A78" s="3">
         <v>77</v>
       </c>
@@ -6743,7 +6808,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="79" spans="1:27" ht="75" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:29" ht="75" x14ac:dyDescent="0.25">
       <c r="A79" s="3">
         <v>78</v>
       </c>
@@ -6799,7 +6864,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="80" spans="1:27" ht="90" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:29" ht="90" x14ac:dyDescent="0.25">
       <c r="A80" s="3">
         <v>79</v>
       </c>
@@ -6846,7 +6911,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="81" spans="1:28" ht="75" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:29" ht="75" x14ac:dyDescent="0.25">
       <c r="A81" s="3">
         <v>80</v>
       </c>
@@ -6886,17 +6951,17 @@
       <c r="P81" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="V81" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="W81" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="X81" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y81" s="8" t="s">
-        <v>89</v>
+      <c r="V81" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="W81" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="X81" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="Y81" s="11" t="s">
+        <v>119</v>
       </c>
       <c r="Z81" s="1" t="s">
         <v>485</v>
@@ -6904,8 +6969,11 @@
       <c r="AA81" s="11" t="s">
         <v>615</v>
       </c>
-    </row>
-    <row r="82" spans="1:28" ht="75" x14ac:dyDescent="0.25">
+      <c r="AC81" s="3" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="82" spans="1:29" ht="90" x14ac:dyDescent="0.25">
       <c r="A82" s="3">
         <v>81</v>
       </c>
@@ -6937,29 +7005,32 @@
       <c r="P82" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="V82" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="W82" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="X82" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y82" s="4" t="s">
-        <v>89</v>
+      <c r="V82" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="W82" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="X82" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="Y82" s="11" t="s">
+        <v>119</v>
       </c>
       <c r="Z82" s="1" t="s">
         <v>490</v>
       </c>
       <c r="AA82" s="11" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
       <c r="AB82" s="1" t="s">
-        <v>645</v>
-      </c>
-    </row>
-    <row r="83" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+        <v>642</v>
+      </c>
+      <c r="AC82" s="1" t="s">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="83" spans="1:29" ht="60" x14ac:dyDescent="0.25">
       <c r="A83" s="3">
         <v>82</v>
       </c>
@@ -6991,23 +7062,26 @@
       <c r="P83" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="V83" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="W83" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="X83" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y83" s="4" t="s">
-        <v>89</v>
+      <c r="V83" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="W83" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="X83" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="Y83" s="11" t="s">
+        <v>119</v>
       </c>
       <c r="AA83" s="11" t="s">
-        <v>644</v>
-      </c>
-    </row>
-    <row r="84" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+        <v>641</v>
+      </c>
+      <c r="AC83" s="1" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="84" spans="1:29" ht="60" x14ac:dyDescent="0.25">
       <c r="A84" s="3">
         <v>83</v>
       </c>
@@ -7039,23 +7113,26 @@
       <c r="P84" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="V84" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="W84" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="X84" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y84" s="4" t="s">
-        <v>89</v>
+      <c r="V84" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="W84" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="X84" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="Y84" s="11" t="s">
+        <v>119</v>
       </c>
       <c r="AA84" s="11" t="s">
-        <v>644</v>
-      </c>
-    </row>
-    <row r="85" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+        <v>641</v>
+      </c>
+      <c r="AC84" s="1" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="85" spans="1:29" ht="60" x14ac:dyDescent="0.25">
       <c r="A85" s="3">
         <v>84</v>
       </c>
@@ -7087,23 +7164,26 @@
       <c r="P85" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="V85" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="W85" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="X85" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y85" s="4" t="s">
-        <v>89</v>
+      <c r="V85" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="W85" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="X85" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="Y85" s="11" t="s">
+        <v>119</v>
       </c>
       <c r="AA85" s="11" t="s">
-        <v>644</v>
-      </c>
-    </row>
-    <row r="86" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+        <v>641</v>
+      </c>
+      <c r="AC85" s="1" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="86" spans="1:29" ht="60" x14ac:dyDescent="0.25">
       <c r="A86" s="3">
         <v>85</v>
       </c>
@@ -7135,23 +7215,26 @@
       <c r="P86" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="V86" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="W86" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="X86" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y86" s="4" t="s">
-        <v>89</v>
+      <c r="V86" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="W86" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="X86" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="Y86" s="11" t="s">
+        <v>119</v>
       </c>
       <c r="AA86" s="11" t="s">
-        <v>644</v>
-      </c>
-    </row>
-    <row r="87" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+        <v>641</v>
+      </c>
+      <c r="AC86" s="1" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="87" spans="1:29" ht="60" x14ac:dyDescent="0.25">
       <c r="A87" s="3">
         <v>86</v>
       </c>
@@ -7183,23 +7266,26 @@
       <c r="P87" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="V87" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="W87" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="X87" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y87" s="4" t="s">
-        <v>89</v>
+      <c r="V87" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="W87" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="X87" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="Y87" s="11" t="s">
+        <v>119</v>
       </c>
       <c r="AA87" s="11" t="s">
-        <v>644</v>
-      </c>
-    </row>
-    <row r="88" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+        <v>641</v>
+      </c>
+      <c r="AC87" s="1" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="88" spans="1:29" ht="60" x14ac:dyDescent="0.25">
       <c r="A88" s="3">
         <v>87</v>
       </c>
@@ -7231,23 +7317,26 @@
       <c r="P88" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="V88" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="W88" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="X88" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y88" s="4" t="s">
-        <v>89</v>
+      <c r="V88" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="W88" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="X88" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="Y88" s="11" t="s">
+        <v>119</v>
       </c>
       <c r="AA88" s="11" t="s">
-        <v>644</v>
-      </c>
-    </row>
-    <row r="89" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+        <v>641</v>
+      </c>
+      <c r="AC88" s="1" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="89" spans="1:29" ht="60" x14ac:dyDescent="0.25">
       <c r="A89" s="3">
         <v>88</v>
       </c>
@@ -7279,23 +7368,26 @@
       <c r="P89" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="V89" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="W89" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="X89" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y89" s="4" t="s">
-        <v>89</v>
+      <c r="V89" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="W89" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="X89" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="Y89" s="11" t="s">
+        <v>119</v>
       </c>
       <c r="AA89" s="11" t="s">
-        <v>644</v>
-      </c>
-    </row>
-    <row r="90" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+        <v>641</v>
+      </c>
+      <c r="AC89" s="1" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="90" spans="1:29" ht="60" x14ac:dyDescent="0.25">
       <c r="A90" s="3">
         <v>89</v>
       </c>
@@ -7327,23 +7419,26 @@
       <c r="P90" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="V90" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="W90" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="X90" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y90" s="4" t="s">
-        <v>89</v>
+      <c r="V90" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="W90" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="X90" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="Y90" s="11" t="s">
+        <v>119</v>
       </c>
       <c r="AA90" s="11" t="s">
-        <v>644</v>
-      </c>
-    </row>
-    <row r="91" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+        <v>641</v>
+      </c>
+      <c r="AC90" s="1" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="91" spans="1:29" ht="60" x14ac:dyDescent="0.25">
       <c r="A91" s="3">
         <v>90</v>
       </c>
@@ -7375,23 +7470,26 @@
       <c r="P91" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="V91" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="W91" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="X91" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y91" s="4" t="s">
-        <v>89</v>
+      <c r="V91" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="W91" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="X91" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="Y91" s="11" t="s">
+        <v>119</v>
       </c>
       <c r="AA91" s="11" t="s">
-        <v>644</v>
-      </c>
-    </row>
-    <row r="92" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+        <v>641</v>
+      </c>
+      <c r="AC91" s="1" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="92" spans="1:29" ht="45" x14ac:dyDescent="0.25">
       <c r="A92" s="3">
         <v>91</v>
       </c>
@@ -7428,17 +7526,17 @@
       <c r="P92" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="V92" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="W92" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="X92" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y92" s="8" t="s">
-        <v>89</v>
+      <c r="V92" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="W92" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="X92" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="Y92" s="11" t="s">
+        <v>119</v>
       </c>
       <c r="Z92" s="1" t="s">
         <v>523</v>
@@ -7446,8 +7544,11 @@
       <c r="AA92" s="11" t="s">
         <v>615</v>
       </c>
-    </row>
-    <row r="93" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+      <c r="AC92" s="3" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="93" spans="1:29" ht="60" x14ac:dyDescent="0.25">
       <c r="A93" s="3">
         <v>92</v>
       </c>
@@ -7479,23 +7580,26 @@
       <c r="P93" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="V93" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="W93" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="X93" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y93" s="4" t="s">
-        <v>89</v>
+      <c r="V93" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="W93" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="X93" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="Y93" s="11" t="s">
+        <v>119</v>
       </c>
       <c r="AA93" s="11" t="s">
-        <v>644</v>
-      </c>
-    </row>
-    <row r="94" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+        <v>641</v>
+      </c>
+      <c r="AC93" s="1" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="94" spans="1:29" ht="60" x14ac:dyDescent="0.25">
       <c r="A94" s="3">
         <v>93</v>
       </c>
@@ -7527,23 +7631,26 @@
       <c r="P94" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="V94" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="W94" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="X94" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y94" s="4" t="s">
-        <v>89</v>
+      <c r="V94" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="W94" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="X94" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="Y94" s="11" t="s">
+        <v>119</v>
       </c>
       <c r="AA94" s="11" t="s">
-        <v>644</v>
-      </c>
-    </row>
-    <row r="95" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+        <v>641</v>
+      </c>
+      <c r="AC94" s="1" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="95" spans="1:29" ht="60" x14ac:dyDescent="0.25">
       <c r="A95" s="3">
         <v>94</v>
       </c>
@@ -7575,23 +7682,26 @@
       <c r="P95" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="V95" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="W95" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="X95" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y95" s="4" t="s">
-        <v>89</v>
+      <c r="V95" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="W95" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="X95" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="Y95" s="11" t="s">
+        <v>119</v>
       </c>
       <c r="AA95" s="11" t="s">
-        <v>644</v>
-      </c>
-    </row>
-    <row r="96" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+        <v>641</v>
+      </c>
+      <c r="AC95" s="1" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="96" spans="1:29" ht="60" x14ac:dyDescent="0.25">
       <c r="A96" s="3">
         <v>95</v>
       </c>
@@ -7623,23 +7733,26 @@
       <c r="P96" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="V96" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="W96" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="X96" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y96" s="4" t="s">
-        <v>89</v>
+      <c r="V96" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="W96" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="X96" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="Y96" s="11" t="s">
+        <v>119</v>
       </c>
       <c r="AA96" s="11" t="s">
-        <v>644</v>
-      </c>
-    </row>
-    <row r="97" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+        <v>641</v>
+      </c>
+      <c r="AC96" s="1" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="97" spans="1:29" ht="60" x14ac:dyDescent="0.25">
       <c r="A97" s="3">
         <v>96</v>
       </c>
@@ -7671,23 +7784,26 @@
       <c r="P97" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="V97" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="W97" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="X97" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y97" s="4" t="s">
-        <v>89</v>
+      <c r="V97" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="W97" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="X97" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="Y97" s="11" t="s">
+        <v>119</v>
       </c>
       <c r="AA97" s="11" t="s">
-        <v>644</v>
-      </c>
-    </row>
-    <row r="98" spans="1:28" x14ac:dyDescent="0.25">
+        <v>641</v>
+      </c>
+      <c r="AC97" s="1" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="98" spans="1:29" ht="60" x14ac:dyDescent="0.25">
       <c r="A98" s="3">
         <v>97</v>
       </c>
@@ -7719,23 +7835,26 @@
       <c r="P98" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="V98" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="W98" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="X98" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y98" s="4" t="s">
-        <v>89</v>
+      <c r="V98" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="W98" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="X98" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="Y98" s="11" t="s">
+        <v>119</v>
       </c>
       <c r="AA98" s="11" t="s">
-        <v>644</v>
-      </c>
-    </row>
-    <row r="99" spans="1:28" x14ac:dyDescent="0.25">
+        <v>641</v>
+      </c>
+      <c r="AC98" s="1" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="99" spans="1:29" ht="60" x14ac:dyDescent="0.25">
       <c r="A99" s="3">
         <v>98</v>
       </c>
@@ -7767,23 +7886,26 @@
       <c r="P99" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="V99" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="W99" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="X99" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y99" s="4" t="s">
-        <v>89</v>
+      <c r="V99" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="W99" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="X99" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="Y99" s="11" t="s">
+        <v>119</v>
       </c>
       <c r="AA99" s="11" t="s">
-        <v>644</v>
-      </c>
-    </row>
-    <row r="100" spans="1:28" x14ac:dyDescent="0.25">
+        <v>641</v>
+      </c>
+      <c r="AC99" s="1" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="100" spans="1:29" ht="60" x14ac:dyDescent="0.25">
       <c r="A100" s="3">
         <v>99</v>
       </c>
@@ -7815,23 +7937,26 @@
       <c r="P100" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="V100" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="W100" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="X100" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y100" s="4" t="s">
-        <v>89</v>
+      <c r="V100" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="W100" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="X100" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="Y100" s="11" t="s">
+        <v>119</v>
       </c>
       <c r="AA100" s="11" t="s">
-        <v>644</v>
-      </c>
-    </row>
-    <row r="101" spans="1:28" x14ac:dyDescent="0.25">
+        <v>641</v>
+      </c>
+      <c r="AC100" s="1" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="101" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A101" s="3">
         <v>100</v>
       </c>
@@ -7876,7 +8001,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="102" spans="1:28" ht="90" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:29" ht="90" x14ac:dyDescent="0.25">
       <c r="A102" s="3">
         <v>101</v>
       </c>
@@ -7905,14 +8030,14 @@
         <v>41</v>
       </c>
       <c r="N102" s="1" t="s">
-        <v>647</v>
+        <v>644</v>
       </c>
       <c r="O102" s="9"/>
       <c r="P102" s="3" t="s">
         <v>32</v>
       </c>
       <c r="T102" s="3" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
       <c r="V102" s="5" t="s">
         <v>89</v>
@@ -7930,10 +8055,10 @@
         <v>556</v>
       </c>
       <c r="AB102" s="11" t="s">
-        <v>646</v>
-      </c>
-    </row>
-    <row r="103" spans="1:28" x14ac:dyDescent="0.25">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="103" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A103" s="3">
         <v>102</v>
       </c>
@@ -7978,7 +8103,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="104" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:29" ht="45" x14ac:dyDescent="0.25">
       <c r="A104" s="3">
         <v>103</v>
       </c>
@@ -8031,7 +8156,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="105" spans="1:28" ht="30" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:29" ht="30" x14ac:dyDescent="0.25">
       <c r="A105" s="3">
         <v>104</v>
       </c>
@@ -8084,7 +8209,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="106" spans="1:28" ht="30" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:29" ht="30" x14ac:dyDescent="0.25">
       <c r="A106" s="3">
         <v>105</v>
       </c>
@@ -8134,7 +8259,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="107" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A107" s="3">
         <v>106</v>
       </c>
@@ -8176,7 +8301,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="108" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A108" s="3">
         <v>107</v>
       </c>
@@ -8218,7 +8343,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="109" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A109" s="3">
         <v>108</v>
       </c>
@@ -8260,7 +8385,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="110" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A110" s="3">
         <v>109</v>
       </c>
@@ -8303,7 +8428,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="111" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:29" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A111" s="3">
         <v>110</v>
       </c>
@@ -8353,7 +8478,7 @@
         <v>596</v>
       </c>
     </row>
-    <row r="112" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A112" s="3">
         <v>111</v>
       </c>
@@ -8447,13 +8572,13 @@
         <v>24</v>
       </c>
       <c r="C114" s="3" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="D114" s="3" t="s">
-        <v>653</v>
+        <v>650</v>
       </c>
       <c r="E114" s="3" t="s">
-        <v>654</v>
+        <v>651</v>
       </c>
       <c r="F114" s="3" t="s">
         <v>51</v>
@@ -8477,7 +8602,7 @@
         <v>89</v>
       </c>
       <c r="AB114" s="1" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
     </row>
     <row r="115" spans="1:28" x14ac:dyDescent="0.25">
@@ -8488,13 +8613,13 @@
         <v>24</v>
       </c>
       <c r="C115" s="3" t="s">
-        <v>650</v>
+        <v>647</v>
       </c>
       <c r="D115" s="3" t="s">
-        <v>655</v>
+        <v>652</v>
       </c>
       <c r="E115" s="3" t="s">
-        <v>655</v>
+        <v>652</v>
       </c>
       <c r="F115" s="3" t="s">
         <v>51</v>
@@ -8518,7 +8643,7 @@
         <v>89</v>
       </c>
       <c r="AB115" s="1" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
     </row>
     <row r="116" spans="1:28" x14ac:dyDescent="0.25">
@@ -8529,13 +8654,13 @@
         <v>24</v>
       </c>
       <c r="C116" s="3" t="s">
-        <v>651</v>
+        <v>648</v>
       </c>
       <c r="D116" s="3" t="s">
-        <v>656</v>
+        <v>653</v>
       </c>
       <c r="E116" s="3" t="s">
-        <v>656</v>
+        <v>653</v>
       </c>
       <c r="F116" s="3" t="s">
         <v>51</v>
@@ -8559,7 +8684,7 @@
         <v>89</v>
       </c>
       <c r="AB116" s="1" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
     </row>
     <row r="117" spans="1:28" x14ac:dyDescent="0.25">
@@ -8570,13 +8695,13 @@
         <v>24</v>
       </c>
       <c r="C117" s="3" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="D117" s="3" t="s">
-        <v>657</v>
+        <v>654</v>
       </c>
       <c r="E117" s="3" t="s">
-        <v>657</v>
+        <v>654</v>
       </c>
       <c r="F117" s="3" t="s">
         <v>51</v>
@@ -8600,7 +8725,7 @@
         <v>89</v>
       </c>
       <c r="AB117" s="1" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Change input_variables to __BLANK__ explicitly
</commit_message>
<xml_diff>
--- a/longitudinal/data_processing_elements_longitudinal-MSN.xlsx
+++ b/longitudinal/data_processing_elements_longitudinal-MSN.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\twey\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A3D4467-982A-46C6-99D5-7EC253F68CC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7595E99-404F-4084-8244-57049F550AAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1688" uniqueCount="661">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1688" uniqueCount="658">
   <si>
     <t>index</t>
   </si>
@@ -1226,10 +1226,6 @@
     <t>1 = Less than once a week ; 
 2 = 1 to 5 times a week ; 
 3 = 6 times or more times a week</t>
-  </si>
-  <si>
-    <t>activity_Q01_freq;
-activity_Q02_frequency</t>
   </si>
   <si>
     <t>Cohort: walking-for-leisure 'same as baseline' (CHAMPS items 'activity_Q01_freq'/'activity_Q02_frequency'); these are not in the longitudinal dictionary - ask if there is a newer version of the data dictionary that has these variables.</t>
@@ -2171,9 +2167,6 @@
     <t>Algorithm based on format of the baseline date, but need to confirm.</t>
   </si>
   <si>
-    <t>N_MajorGroup_ISCO08</t>
-  </si>
-  <si>
     <t>Major Group of ISCO-08</t>
   </si>
   <si>
@@ -2258,14 +2251,6 @@
   </si>
   <si>
     <t>Would it be reasonable to consider these variables as walking for leisure (not transport)? Can details about the format/data types for the variable be provided? If integer/numeric, should be able to harmonize based on summing the two variables. Are missing values coded? Confirm if available in follow-up. If so, confirm variable names.</t>
-  </si>
-  <si>
-    <t>activity_Q04_done ; 
-activity_Q09_done ; 
-activity_Q10_done ; 
-activity_Q11_done ; 
-activity_Q12_done ; 
-activity_Q14_done</t>
   </si>
   <si>
     <t>fast cycling past 4 weeks ; 
@@ -2807,6 +2792,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:AF113"/>
   <sheetFormatPr defaultColWidth="28.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2896,7 +2882,7 @@
         <v>19</v>
       </c>
       <c r="U1" s="2" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="V1" s="2" t="s">
         <v>20</v>
@@ -2911,28 +2897,28 @@
         <v>23</v>
       </c>
       <c r="Z1" s="12" t="s">
+        <v>599</v>
+      </c>
+      <c r="AA1" s="2" t="s">
         <v>600</v>
       </c>
-      <c r="AA1" s="2" t="s">
+      <c r="AB1" s="2" t="s">
         <v>601</v>
       </c>
-      <c r="AB1" s="2" t="s">
+      <c r="AC1" s="2" t="s">
         <v>602</v>
       </c>
-      <c r="AC1" s="2" t="s">
+      <c r="AD1" s="2" t="s">
         <v>603</v>
       </c>
-      <c r="AD1" s="2" t="s">
+      <c r="AE1" s="2" t="s">
         <v>604</v>
       </c>
-      <c r="AE1" s="2" t="s">
+      <c r="AF1" s="2" t="s">
         <v>605</v>
       </c>
-      <c r="AF1" s="2" t="s">
-        <v>606</v>
-      </c>
-    </row>
-    <row r="2" spans="1:32" ht="75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:32" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -2955,7 +2941,7 @@
         <v>29</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>660</v>
+        <v>657</v>
       </c>
       <c r="N2" s="3" t="s">
         <v>30</v>
@@ -2973,13 +2959,13 @@
         <v>34</v>
       </c>
       <c r="Y2" s="4" t="s">
-        <v>660</v>
+        <v>657</v>
       </c>
       <c r="Z2" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:32" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -3020,7 +3006,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:32" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -3061,7 +3047,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:32" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -3102,7 +3088,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:32" ht="60" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:32" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -3158,13 +3144,13 @@
         <v>64</v>
       </c>
       <c r="AA6" s="11" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="AC6" s="3" t="s">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="7" spans="1:32" ht="30" x14ac:dyDescent="0.25">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="7" spans="1:32" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -3211,7 +3197,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="8" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:32" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -3264,7 +3250,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="9" spans="1:32" ht="165" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:32" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -3308,7 +3294,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="10" spans="1:32" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:32" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>9</v>
       </c>
@@ -3352,7 +3338,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="11" spans="1:32" ht="90" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:32" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -3402,7 +3388,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="12" spans="1:32" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:32" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>11</v>
       </c>
@@ -3449,7 +3435,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="13" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:32" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -3510,19 +3496,19 @@
         <v>28</v>
       </c>
       <c r="M14" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="N14" s="3" t="s">
+        <v>607</v>
+      </c>
+      <c r="O14" s="1" t="s">
         <v>608</v>
       </c>
-      <c r="N14" s="3" t="s">
-        <v>609</v>
-      </c>
-      <c r="O14" s="1" t="s">
-        <v>610</v>
-      </c>
       <c r="P14" s="3" t="s">
         <v>31</v>
       </c>
       <c r="U14" s="3" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="V14" s="5" t="s">
         <v>88</v>
@@ -3540,16 +3526,16 @@
         <v>117</v>
       </c>
       <c r="AA14" s="11" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="AB14" s="1" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="AC14" s="3" t="s">
-        <v>651</v>
-      </c>
-    </row>
-    <row r="15" spans="1:32" ht="75" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="15" spans="1:32" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -3599,7 +3585,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="16" spans="1:32" ht="135" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:32" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>15</v>
       </c>
@@ -3646,7 +3632,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>16</v>
       </c>
@@ -3693,7 +3679,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="18" spans="1:28" ht="60" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:28" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>17</v>
       </c>
@@ -3743,7 +3729,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="19" spans="1:28" ht="60" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:28" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -3787,7 +3773,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="20" spans="1:28" ht="60" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:28" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>19</v>
       </c>
@@ -3837,7 +3823,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="21" spans="1:28" ht="60" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:28" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>20</v>
       </c>
@@ -3881,7 +3867,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="22" spans="1:28" ht="60" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:28" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
         <v>21</v>
       </c>
@@ -3932,7 +3918,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="23" spans="1:28" ht="60" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:28" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>22</v>
       </c>
@@ -3961,7 +3947,7 @@
         <v>145</v>
       </c>
       <c r="M23" s="1" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
       <c r="N23" s="3" t="s">
         <v>173</v>
@@ -3982,10 +3968,10 @@
         <v>174</v>
       </c>
       <c r="AB23" s="1" t="s">
-        <v>646</v>
-      </c>
-    </row>
-    <row r="24" spans="1:28" ht="60" x14ac:dyDescent="0.25">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="24" spans="1:28" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
         <v>23</v>
       </c>
@@ -4008,7 +3994,7 @@
         <v>151</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
       <c r="N24" s="3" t="s">
         <v>173</v>
@@ -4029,10 +4015,10 @@
         <v>177</v>
       </c>
       <c r="AB24" s="1" t="s">
-        <v>646</v>
-      </c>
-    </row>
-    <row r="25" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="25" spans="1:28" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>24</v>
       </c>
@@ -4076,7 +4062,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="26" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:28" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3">
         <v>25</v>
       </c>
@@ -4117,7 +4103,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="27" spans="1:28" ht="60" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:28" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3">
         <v>26</v>
       </c>
@@ -4167,7 +4153,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="28" spans="1:28" ht="60" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:28" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3">
         <v>27</v>
       </c>
@@ -4217,7 +4203,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="29" spans="1:28" ht="60" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:28" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3">
         <v>28</v>
       </c>
@@ -4267,7 +4253,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="30" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:28" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3">
         <v>29</v>
       </c>
@@ -4317,7 +4303,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="31" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3">
         <v>30</v>
       </c>
@@ -4358,7 +4344,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="32" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3">
         <v>31</v>
       </c>
@@ -4400,7 +4386,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="33" spans="1:28" ht="60" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:28" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
         <v>32</v>
       </c>
@@ -4444,7 +4430,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="34" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:28" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3">
         <v>33</v>
       </c>
@@ -4489,7 +4475,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="35" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:28" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
         <v>34</v>
       </c>
@@ -4533,7 +4519,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="36" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:28" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
         <v>35</v>
       </c>
@@ -4577,7 +4563,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="37" spans="1:28" ht="90" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:28" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
         <v>36</v>
       </c>
@@ -4625,10 +4611,10 @@
         <v>247</v>
       </c>
       <c r="AB37" s="1" t="s">
-        <v>647</v>
-      </c>
-    </row>
-    <row r="38" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="38" spans="1:28" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="3">
         <v>37</v>
       </c>
@@ -4673,7 +4659,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="39" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:28" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="3">
         <v>38</v>
       </c>
@@ -4718,7 +4704,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="40" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:28" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="3">
         <v>39</v>
       </c>
@@ -4770,7 +4756,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="41" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:28" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="3">
         <v>40</v>
       </c>
@@ -4818,7 +4804,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="42" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:28" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="3">
         <v>41</v>
       </c>
@@ -4870,7 +4856,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="43" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:28" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="3">
         <v>42</v>
       </c>
@@ -4921,7 +4907,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="44" spans="1:28" ht="60" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:28" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3">
         <v>43</v>
       </c>
@@ -4972,7 +4958,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="45" spans="1:28" ht="60" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:28" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="3">
         <v>44</v>
       </c>
@@ -5023,16 +5009,16 @@
         <v>102</v>
       </c>
       <c r="Y45" s="4" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="Z45" s="1" t="s">
         <v>288</v>
       </c>
       <c r="AB45" s="1" t="s">
-        <v>648</v>
-      </c>
-    </row>
-    <row r="46" spans="1:28" ht="60" x14ac:dyDescent="0.25">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="46" spans="1:28" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="3">
         <v>45</v>
       </c>
@@ -5077,7 +5063,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="47" spans="1:28" ht="135" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:28" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="3">
         <v>46</v>
       </c>
@@ -5130,7 +5116,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="48" spans="1:28" ht="90" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:28" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="3">
         <v>47</v>
       </c>
@@ -5178,10 +5164,10 @@
         <v>304</v>
       </c>
       <c r="AB48" s="1" t="s">
-        <v>612</v>
-      </c>
-    </row>
-    <row r="49" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="49" spans="1:29" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3">
         <v>48</v>
       </c>
@@ -5236,16 +5222,16 @@
         <v>310</v>
       </c>
       <c r="AA49" s="11" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="AB49" s="1" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="AC49" s="3" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="50" spans="1:29" x14ac:dyDescent="0.25">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="50" spans="1:29" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="3">
         <v>49</v>
       </c>
@@ -5316,25 +5302,25 @@
         <v>317</v>
       </c>
       <c r="N51" s="3" t="s">
+        <v>614</v>
+      </c>
+      <c r="O51" s="9" t="s">
+        <v>615</v>
+      </c>
+      <c r="P51" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="T51" s="3" t="s">
         <v>616</v>
       </c>
-      <c r="O51" s="9" t="s">
+      <c r="U51" s="3" t="s">
+        <v>620</v>
+      </c>
+      <c r="V51" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="W51" s="5" t="s">
         <v>617</v>
-      </c>
-      <c r="P51" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="T51" s="3" t="s">
-        <v>618</v>
-      </c>
-      <c r="U51" s="3" t="s">
-        <v>622</v>
-      </c>
-      <c r="V51" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="W51" s="5" t="s">
-        <v>619</v>
       </c>
       <c r="X51" s="5" t="s">
         <v>88</v>
@@ -5346,7 +5332,7 @@
         <v>318</v>
       </c>
       <c r="AB51" s="1" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
     </row>
     <row r="52" spans="1:29" ht="75" x14ac:dyDescent="0.25">
@@ -5375,22 +5361,22 @@
         <v>323</v>
       </c>
       <c r="M52" s="1" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="N52" s="3" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="O52" s="9" t="s">
+        <v>621</v>
+      </c>
+      <c r="P52" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="T52" s="3" t="s">
         <v>623</v>
       </c>
-      <c r="P52" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="T52" s="3" t="s">
+      <c r="U52" s="3" t="s">
         <v>625</v>
-      </c>
-      <c r="U52" s="3" t="s">
-        <v>627</v>
       </c>
       <c r="V52" s="5" t="s">
         <v>118</v>
@@ -5408,16 +5394,16 @@
         <v>324</v>
       </c>
       <c r="AA52" s="11" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="AB52" s="1" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="AC52" s="1" t="s">
-        <v>654</v>
-      </c>
-    </row>
-    <row r="53" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="53" spans="1:29" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="3">
         <v>52</v>
       </c>
@@ -5465,7 +5451,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="54" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:29" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="3">
         <v>53</v>
       </c>
@@ -5510,7 +5496,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="55" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:29" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="3">
         <v>54</v>
       </c>
@@ -5555,7 +5541,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="56" spans="1:29" ht="315" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:29" ht="315" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3">
         <v>55</v>
       </c>
@@ -5600,7 +5586,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="57" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:29" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" s="3">
         <v>56</v>
       </c>
@@ -5648,7 +5634,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="58" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:29" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="3">
         <v>57</v>
       </c>
@@ -5697,7 +5683,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="59" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:29" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="3">
         <v>58</v>
       </c>
@@ -5746,7 +5732,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="60" spans="1:29" ht="135" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:29" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="3">
         <v>59</v>
       </c>
@@ -5817,17 +5803,17 @@
         <v>353</v>
       </c>
       <c r="M61" s="11" t="s">
-        <v>354</v>
+        <v>40</v>
       </c>
       <c r="N61" s="1" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
       <c r="O61" s="11"/>
       <c r="P61" s="3" t="s">
         <v>31</v>
       </c>
       <c r="T61" s="3" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="V61" s="5" t="s">
         <v>118</v>
@@ -5842,19 +5828,19 @@
         <v>118</v>
       </c>
       <c r="Z61" s="1" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="AA61" s="11" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="AB61" s="1" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="AC61" s="3" t="s">
-        <v>655</v>
-      </c>
-    </row>
-    <row r="62" spans="1:29" ht="105" x14ac:dyDescent="0.25">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="62" spans="1:29" ht="105" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="3">
         <v>61</v>
       </c>
@@ -5862,13 +5848,13 @@
         <v>24</v>
       </c>
       <c r="C62" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="D62" s="3" t="s">
         <v>356</v>
       </c>
-      <c r="D62" s="3" t="s">
+      <c r="E62" s="3" t="s">
         <v>357</v>
-      </c>
-      <c r="E62" s="3" t="s">
-        <v>358</v>
       </c>
       <c r="F62" s="3" t="s">
         <v>50</v>
@@ -5877,7 +5863,7 @@
         <v>352</v>
       </c>
       <c r="L62" s="1" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="M62" s="1" t="s">
         <v>40</v>
@@ -5907,19 +5893,19 @@
         <v>24</v>
       </c>
       <c r="C63" s="3" t="s">
+        <v>359</v>
+      </c>
+      <c r="D63" s="3" t="s">
         <v>360</v>
       </c>
-      <c r="D63" s="3" t="s">
+      <c r="E63" s="3" t="s">
         <v>361</v>
-      </c>
-      <c r="E63" s="3" t="s">
-        <v>362</v>
       </c>
       <c r="F63" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J63" s="3" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="K63" s="3" t="s">
         <v>352</v>
@@ -5928,19 +5914,19 @@
         <v>93</v>
       </c>
       <c r="M63" s="11" t="s">
-        <v>635</v>
+        <v>40</v>
       </c>
       <c r="N63" s="1" t="s">
-        <v>636</v>
+        <v>633</v>
       </c>
       <c r="O63" s="1" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="P63" s="3" t="s">
         <v>31</v>
       </c>
       <c r="T63" s="3" t="s">
-        <v>637</v>
+        <v>634</v>
       </c>
       <c r="U63" s="11"/>
       <c r="V63" s="11" t="s">
@@ -5956,19 +5942,19 @@
         <v>118</v>
       </c>
       <c r="Z63" s="1" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="AA63" s="11" t="s">
-        <v>638</v>
+        <v>635</v>
       </c>
       <c r="AB63" s="1" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="AC63" s="1" t="s">
-        <v>656</v>
-      </c>
-    </row>
-    <row r="64" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="64" spans="1:29" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="3">
         <v>63</v>
       </c>
@@ -5976,19 +5962,19 @@
         <v>24</v>
       </c>
       <c r="C64" s="3" t="s">
+        <v>364</v>
+      </c>
+      <c r="D64" s="3" t="s">
         <v>365</v>
       </c>
-      <c r="D64" s="3" t="s">
+      <c r="E64" s="3" t="s">
         <v>366</v>
-      </c>
-      <c r="E64" s="3" t="s">
-        <v>367</v>
       </c>
       <c r="F64" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J64" s="3" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="L64" s="1" t="s">
         <v>93</v>
@@ -6013,7 +5999,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="65" spans="1:29" ht="60" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:29" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3">
         <v>64</v>
       </c>
@@ -6021,19 +6007,19 @@
         <v>24</v>
       </c>
       <c r="C65" s="3" t="s">
+        <v>368</v>
+      </c>
+      <c r="D65" s="3" t="s">
         <v>369</v>
       </c>
-      <c r="D65" s="3" t="s">
+      <c r="E65" s="3" t="s">
         <v>370</v>
-      </c>
-      <c r="E65" s="3" t="s">
-        <v>371</v>
       </c>
       <c r="F65" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J65" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="K65" s="3" t="s">
         <v>352</v>
@@ -6042,10 +6028,10 @@
         <v>93</v>
       </c>
       <c r="M65" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="N65" s="3" t="s">
         <v>373</v>
-      </c>
-      <c r="N65" s="3" t="s">
-        <v>374</v>
       </c>
       <c r="O65" s="9"/>
       <c r="P65" s="3" t="s">
@@ -6061,10 +6047,10 @@
         <v>102</v>
       </c>
       <c r="Y65" s="4" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="66" spans="1:29" ht="409.5" x14ac:dyDescent="0.25">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="66" spans="1:29" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="3">
         <v>65</v>
       </c>
@@ -6072,29 +6058,29 @@
         <v>24</v>
       </c>
       <c r="C66" s="3" t="s">
+        <v>375</v>
+      </c>
+      <c r="D66" s="3" t="s">
         <v>376</v>
       </c>
-      <c r="D66" s="3" t="s">
+      <c r="E66" s="3" t="s">
         <v>377</v>
-      </c>
-      <c r="E66" s="3" t="s">
-        <v>378</v>
       </c>
       <c r="F66" s="3" t="s">
         <v>112</v>
       </c>
       <c r="J66" s="3" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="L66" s="1"/>
       <c r="M66" s="1" t="s">
+        <v>379</v>
+      </c>
+      <c r="N66" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="N66" s="1" t="s">
+      <c r="O66" s="1" t="s">
         <v>381</v>
-      </c>
-      <c r="O66" s="1" t="s">
-        <v>382</v>
       </c>
       <c r="P66" s="3" t="s">
         <v>31</v>
@@ -6109,13 +6095,13 @@
         <v>62</v>
       </c>
       <c r="Y66" s="4" t="s">
+        <v>382</v>
+      </c>
+      <c r="Z66" s="1" t="s">
         <v>383</v>
       </c>
-      <c r="Z66" s="1" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="67" spans="1:29" ht="409.5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="67" spans="1:29" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="3">
         <v>66</v>
       </c>
@@ -6123,29 +6109,29 @@
         <v>24</v>
       </c>
       <c r="C67" s="3" t="s">
+        <v>384</v>
+      </c>
+      <c r="D67" s="3" t="s">
         <v>385</v>
       </c>
-      <c r="D67" s="3" t="s">
+      <c r="E67" s="3" t="s">
         <v>386</v>
-      </c>
-      <c r="E67" s="3" t="s">
-        <v>387</v>
       </c>
       <c r="F67" s="3" t="s">
         <v>50</v>
       </c>
       <c r="G67" s="3" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="L67" s="1"/>
       <c r="M67" s="1" t="s">
+        <v>379</v>
+      </c>
+      <c r="N67" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="N67" s="1" t="s">
+      <c r="O67" s="1" t="s">
         <v>381</v>
-      </c>
-      <c r="O67" s="1" t="s">
-        <v>382</v>
       </c>
       <c r="P67" s="3" t="s">
         <v>31</v>
@@ -6160,13 +6146,13 @@
         <v>62</v>
       </c>
       <c r="Y67" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="Z67" s="1" t="s">
         <v>389</v>
       </c>
-      <c r="Z67" s="1" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="68" spans="1:29" ht="75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="68" spans="1:29" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="3">
         <v>67</v>
       </c>
@@ -6174,31 +6160,31 @@
         <v>24</v>
       </c>
       <c r="C68" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="D68" s="3" t="s">
         <v>391</v>
       </c>
-      <c r="D68" s="3" t="s">
-        <v>392</v>
-      </c>
       <c r="E68" s="3" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="F68" s="3" t="s">
         <v>50</v>
       </c>
       <c r="K68" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="L68" s="1" t="s">
         <v>393</v>
       </c>
-      <c r="L68" s="1" t="s">
+      <c r="M68" s="1" t="s">
         <v>394</v>
       </c>
-      <c r="M68" s="1" t="s">
+      <c r="N68" s="3" t="s">
         <v>395</v>
       </c>
-      <c r="N68" s="3" t="s">
+      <c r="O68" s="1" t="s">
         <v>396</v>
-      </c>
-      <c r="O68" s="1" t="s">
-        <v>397</v>
       </c>
       <c r="P68" s="3" t="s">
         <v>31</v>
@@ -6213,10 +6199,10 @@
         <v>71</v>
       </c>
       <c r="Y68" s="4" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="69" spans="1:29" ht="165" x14ac:dyDescent="0.25">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="69" spans="1:29" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="3">
         <v>68</v>
       </c>
@@ -6224,34 +6210,34 @@
         <v>24</v>
       </c>
       <c r="C69" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="D69" s="3" t="s">
         <v>399</v>
       </c>
-      <c r="D69" s="3" t="s">
+      <c r="E69" s="3" t="s">
         <v>400</v>
-      </c>
-      <c r="E69" s="3" t="s">
-        <v>401</v>
       </c>
       <c r="F69" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J69" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="K69" s="3" t="s">
         <v>402</v>
       </c>
-      <c r="K69" s="3" t="s">
+      <c r="L69" s="1" t="s">
         <v>403</v>
       </c>
-      <c r="L69" s="1" t="s">
+      <c r="M69" s="8" t="s">
         <v>404</v>
       </c>
-      <c r="M69" s="8" t="s">
+      <c r="N69" s="1" t="s">
         <v>405</v>
       </c>
-      <c r="N69" s="1" t="s">
+      <c r="O69" s="1" t="s">
         <v>406</v>
-      </c>
-      <c r="O69" s="1" t="s">
-        <v>407</v>
       </c>
       <c r="P69" s="3" t="s">
         <v>31</v>
@@ -6266,13 +6252,13 @@
         <v>102</v>
       </c>
       <c r="Y69" s="4" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="Z69" s="1" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="70" spans="1:29" ht="75" x14ac:dyDescent="0.25">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="70" spans="1:29" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="3">
         <v>69</v>
       </c>
@@ -6280,25 +6266,25 @@
         <v>24</v>
       </c>
       <c r="C70" s="3" t="s">
+        <v>409</v>
+      </c>
+      <c r="D70" s="3" t="s">
         <v>410</v>
       </c>
-      <c r="D70" s="3" t="s">
+      <c r="E70" s="3" t="s">
         <v>411</v>
-      </c>
-      <c r="E70" s="3" t="s">
-        <v>412</v>
       </c>
       <c r="F70" s="3" t="s">
         <v>50</v>
       </c>
       <c r="I70" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="J70" s="3" t="s">
         <v>413</v>
       </c>
-      <c r="J70" s="3" t="s">
-        <v>414</v>
-      </c>
       <c r="L70" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M70" s="1" t="s">
         <v>40</v>
@@ -6320,16 +6306,16 @@
         <v>118</v>
       </c>
       <c r="Z70" s="1" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="AA70" s="11" t="s">
-        <v>639</v>
+        <v>636</v>
       </c>
       <c r="AC70" s="3" t="s">
-        <v>657</v>
-      </c>
-    </row>
-    <row r="71" spans="1:29" ht="75" x14ac:dyDescent="0.25">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="71" spans="1:29" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="3">
         <v>70</v>
       </c>
@@ -6337,61 +6323,61 @@
         <v>24</v>
       </c>
       <c r="C71" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="D71" s="3" t="s">
         <v>416</v>
       </c>
-      <c r="D71" s="3" t="s">
+      <c r="E71" s="3" t="s">
         <v>417</v>
-      </c>
-      <c r="E71" s="3" t="s">
-        <v>418</v>
       </c>
       <c r="F71" s="3" t="s">
         <v>50</v>
       </c>
       <c r="I71" s="3" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="J71" s="3" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="L71" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M71" s="8" t="s">
         <v>40</v>
       </c>
       <c r="N71" s="3" t="s">
+        <v>419</v>
+      </c>
+      <c r="O71" s="9" t="s">
         <v>420</v>
       </c>
-      <c r="O71" s="9" t="s">
+      <c r="P71" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="V71" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="W71" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="X71" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="Y71" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="Z71" s="1" t="s">
         <v>421</v>
       </c>
-      <c r="P71" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="V71" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="W71" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="X71" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="Y71" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="Z71" s="1" t="s">
-        <v>422</v>
-      </c>
       <c r="AA71" s="11" t="s">
-        <v>639</v>
+        <v>636</v>
       </c>
       <c r="AC71" s="3" t="s">
-        <v>657</v>
-      </c>
-    </row>
-    <row r="72" spans="1:29" ht="75" x14ac:dyDescent="0.25">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="72" spans="1:29" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="3">
         <v>71</v>
       </c>
@@ -6399,61 +6385,61 @@
         <v>24</v>
       </c>
       <c r="C72" s="3" t="s">
+        <v>422</v>
+      </c>
+      <c r="D72" s="3" t="s">
         <v>423</v>
       </c>
-      <c r="D72" s="3" t="s">
+      <c r="E72" s="3" t="s">
         <v>424</v>
-      </c>
-      <c r="E72" s="3" t="s">
-        <v>425</v>
       </c>
       <c r="F72" s="3" t="s">
         <v>50</v>
       </c>
       <c r="I72" s="3" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="J72" s="3" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="L72" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M72" s="8" t="s">
         <v>40</v>
       </c>
       <c r="N72" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="O72" s="9" t="s">
         <v>427</v>
       </c>
-      <c r="O72" s="9" t="s">
+      <c r="P72" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="V72" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="W72" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="X72" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="Y72" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="Z72" s="1" t="s">
         <v>428</v>
       </c>
-      <c r="P72" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="V72" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="W72" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="X72" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="Y72" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="Z72" s="1" t="s">
-        <v>429</v>
-      </c>
       <c r="AA72" s="11" t="s">
-        <v>639</v>
+        <v>636</v>
       </c>
       <c r="AC72" s="3" t="s">
-        <v>657</v>
-      </c>
-    </row>
-    <row r="73" spans="1:29" ht="75" x14ac:dyDescent="0.25">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="73" spans="1:29" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" s="3">
         <v>72</v>
       </c>
@@ -6461,61 +6447,61 @@
         <v>24</v>
       </c>
       <c r="C73" s="3" t="s">
+        <v>429</v>
+      </c>
+      <c r="D73" s="3" t="s">
         <v>430</v>
       </c>
-      <c r="D73" s="3" t="s">
+      <c r="E73" s="3" t="s">
         <v>431</v>
-      </c>
-      <c r="E73" s="3" t="s">
-        <v>432</v>
       </c>
       <c r="F73" s="3" t="s">
         <v>50</v>
       </c>
       <c r="I73" s="3" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="J73" s="3" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="L73" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M73" s="8" t="s">
         <v>40</v>
       </c>
       <c r="N73" s="3" t="s">
+        <v>433</v>
+      </c>
+      <c r="O73" s="9" t="s">
+        <v>420</v>
+      </c>
+      <c r="P73" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="V73" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="W73" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="X73" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="Y73" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="Z73" s="1" t="s">
         <v>434</v>
       </c>
-      <c r="O73" s="9" t="s">
-        <v>421</v>
-      </c>
-      <c r="P73" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="V73" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="W73" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="X73" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="Y73" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="Z73" s="1" t="s">
-        <v>435</v>
-      </c>
       <c r="AA73" s="11" t="s">
-        <v>639</v>
+        <v>636</v>
       </c>
       <c r="AC73" s="3" t="s">
-        <v>657</v>
-      </c>
-    </row>
-    <row r="74" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="74" spans="1:29" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="3">
         <v>73</v>
       </c>
@@ -6523,25 +6509,25 @@
         <v>24</v>
       </c>
       <c r="C74" s="3" t="s">
+        <v>435</v>
+      </c>
+      <c r="D74" s="3" t="s">
         <v>436</v>
       </c>
-      <c r="D74" s="3" t="s">
+      <c r="E74" s="3" t="s">
         <v>437</v>
-      </c>
-      <c r="E74" s="3" t="s">
-        <v>438</v>
       </c>
       <c r="F74" s="3" t="s">
         <v>50</v>
       </c>
       <c r="I74" s="3" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="J74" s="3" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="L74" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M74" s="1" t="s">
         <v>40</v>
@@ -6563,7 +6549,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="75" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:29" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="3">
         <v>74</v>
       </c>
@@ -6571,25 +6557,25 @@
         <v>24</v>
       </c>
       <c r="C75" s="3" t="s">
+        <v>439</v>
+      </c>
+      <c r="D75" s="3" t="s">
         <v>440</v>
       </c>
-      <c r="D75" s="3" t="s">
+      <c r="E75" s="3" t="s">
         <v>441</v>
-      </c>
-      <c r="E75" s="3" t="s">
-        <v>442</v>
       </c>
       <c r="F75" s="3" t="s">
         <v>50</v>
       </c>
       <c r="I75" s="3" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="J75" s="3" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="L75" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M75" s="1" t="s">
         <v>40</v>
@@ -6611,7 +6597,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="76" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:29" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="3">
         <v>75</v>
       </c>
@@ -6619,28 +6605,28 @@
         <v>24</v>
       </c>
       <c r="C76" s="3" t="s">
+        <v>443</v>
+      </c>
+      <c r="D76" s="3" t="s">
         <v>444</v>
       </c>
-      <c r="D76" s="3" t="s">
+      <c r="E76" s="3" t="s">
         <v>445</v>
-      </c>
-      <c r="E76" s="3" t="s">
-        <v>446</v>
       </c>
       <c r="F76" s="3" t="s">
         <v>50</v>
       </c>
       <c r="I76" s="3" t="s">
+        <v>446</v>
+      </c>
+      <c r="J76" s="3" t="s">
         <v>447</v>
       </c>
-      <c r="J76" s="3" t="s">
+      <c r="K76" s="3" t="s">
         <v>448</v>
       </c>
-      <c r="K76" s="3" t="s">
-        <v>449</v>
-      </c>
       <c r="L76" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M76" s="1" t="s">
         <v>40</v>
@@ -6662,16 +6648,16 @@
         <v>118</v>
       </c>
       <c r="Z76" s="1" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="AA76" s="11" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="AC76" s="3" t="s">
-        <v>657</v>
-      </c>
-    </row>
-    <row r="77" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="77" spans="1:29" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" s="3">
         <v>76</v>
       </c>
@@ -6679,61 +6665,61 @@
         <v>24</v>
       </c>
       <c r="C77" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="D77" s="3" t="s">
         <v>451</v>
       </c>
-      <c r="D77" s="3" t="s">
+      <c r="E77" s="3" t="s">
         <v>452</v>
-      </c>
-      <c r="E77" s="3" t="s">
-        <v>453</v>
       </c>
       <c r="F77" s="3" t="s">
         <v>50</v>
       </c>
       <c r="I77" s="3" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="J77" s="3" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="L77" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M77" s="8" t="s">
         <v>40</v>
       </c>
       <c r="N77" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="O77" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="O77" s="1" t="s">
+      <c r="P77" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="V77" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="W77" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="X77" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="Y77" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="Z77" s="1" t="s">
         <v>456</v>
       </c>
-      <c r="P77" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="V77" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="W77" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="X77" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="Y77" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="Z77" s="1" t="s">
-        <v>457</v>
-      </c>
       <c r="AA77" s="11" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="AC77" s="3" t="s">
-        <v>657</v>
-      </c>
-    </row>
-    <row r="78" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="78" spans="1:29" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" s="3">
         <v>77</v>
       </c>
@@ -6741,22 +6727,22 @@
         <v>24</v>
       </c>
       <c r="C78" s="3" t="s">
+        <v>457</v>
+      </c>
+      <c r="D78" s="3" t="s">
         <v>458</v>
       </c>
-      <c r="D78" s="3" t="s">
+      <c r="E78" s="3" t="s">
         <v>459</v>
-      </c>
-      <c r="E78" s="3" t="s">
-        <v>460</v>
       </c>
       <c r="F78" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J78" s="3" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="L78" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M78" s="1" t="s">
         <v>40</v>
@@ -6778,7 +6764,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="79" spans="1:29" ht="75" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:29" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" s="3">
         <v>78</v>
       </c>
@@ -6786,37 +6772,37 @@
         <v>24</v>
       </c>
       <c r="C79" s="3" t="s">
+        <v>461</v>
+      </c>
+      <c r="D79" s="3" t="s">
         <v>462</v>
       </c>
-      <c r="D79" s="3" t="s">
+      <c r="E79" s="3" t="s">
         <v>463</v>
-      </c>
-      <c r="E79" s="3" t="s">
-        <v>464</v>
       </c>
       <c r="F79" s="3" t="s">
         <v>50</v>
       </c>
       <c r="I79" s="3" t="s">
+        <v>464</v>
+      </c>
+      <c r="J79" s="3" t="s">
+        <v>460</v>
+      </c>
+      <c r="K79" s="3" t="s">
         <v>465</v>
       </c>
-      <c r="J79" s="3" t="s">
-        <v>461</v>
-      </c>
-      <c r="K79" s="3" t="s">
+      <c r="L79" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="M79" s="1" t="s">
         <v>466</v>
       </c>
-      <c r="L79" s="1" t="s">
-        <v>404</v>
-      </c>
-      <c r="M79" s="1" t="s">
+      <c r="N79" s="3" t="s">
         <v>467</v>
       </c>
-      <c r="N79" s="3" t="s">
+      <c r="O79" s="1" t="s">
         <v>468</v>
-      </c>
-      <c r="O79" s="1" t="s">
-        <v>469</v>
       </c>
       <c r="P79" s="3" t="s">
         <v>31</v>
@@ -6831,10 +6817,10 @@
         <v>71</v>
       </c>
       <c r="Y79" s="4" t="s">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="80" spans="1:29" ht="90" x14ac:dyDescent="0.25">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="80" spans="1:29" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" s="3">
         <v>79</v>
       </c>
@@ -6842,28 +6828,28 @@
         <v>24</v>
       </c>
       <c r="C80" s="3" t="s">
+        <v>470</v>
+      </c>
+      <c r="D80" s="3" t="s">
         <v>471</v>
       </c>
-      <c r="D80" s="3" t="s">
-        <v>472</v>
-      </c>
       <c r="E80" s="3" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="F80" s="3" t="s">
         <v>50</v>
       </c>
       <c r="K80" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="L80" s="1" t="s">
         <v>473</v>
       </c>
-      <c r="L80" s="1" t="s">
+      <c r="M80" s="1" t="s">
+        <v>466</v>
+      </c>
+      <c r="O80" s="1" t="s">
         <v>474</v>
-      </c>
-      <c r="M80" s="1" t="s">
-        <v>467</v>
-      </c>
-      <c r="O80" s="1" t="s">
-        <v>475</v>
       </c>
       <c r="P80" s="3" t="s">
         <v>31</v>
@@ -6878,10 +6864,10 @@
         <v>71</v>
       </c>
       <c r="Y80" s="4" t="s">
-        <v>476</v>
-      </c>
-    </row>
-    <row r="81" spans="1:29" ht="75" x14ac:dyDescent="0.25">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="81" spans="1:29" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" s="3">
         <v>80</v>
       </c>
@@ -6889,61 +6875,61 @@
         <v>24</v>
       </c>
       <c r="C81" s="3" t="s">
+        <v>476</v>
+      </c>
+      <c r="D81" s="3" t="s">
         <v>477</v>
       </c>
-      <c r="D81" s="3" t="s">
+      <c r="E81" s="3" t="s">
         <v>478</v>
-      </c>
-      <c r="E81" s="3" t="s">
-        <v>479</v>
       </c>
       <c r="F81" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J81" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="K81" s="3" t="s">
         <v>480</v>
       </c>
-      <c r="K81" s="3" t="s">
-        <v>481</v>
-      </c>
       <c r="L81" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M81" s="8" t="s">
         <v>40</v>
       </c>
       <c r="N81" s="1" t="s">
+        <v>481</v>
+      </c>
+      <c r="O81" s="9" t="s">
         <v>482</v>
       </c>
-      <c r="O81" s="9" t="s">
+      <c r="P81" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="V81" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="W81" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="X81" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="Y81" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="Z81" s="1" t="s">
         <v>483</v>
       </c>
-      <c r="P81" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="V81" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="W81" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="X81" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="Y81" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="Z81" s="1" t="s">
-        <v>484</v>
-      </c>
       <c r="AA81" s="11" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="AC81" s="3" t="s">
-        <v>657</v>
-      </c>
-    </row>
-    <row r="82" spans="1:29" ht="90" x14ac:dyDescent="0.25">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="82" spans="1:29" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3">
         <v>81</v>
       </c>
@@ -6951,22 +6937,22 @@
         <v>24</v>
       </c>
       <c r="C82" s="3" t="s">
+        <v>484</v>
+      </c>
+      <c r="D82" s="3" t="s">
         <v>485</v>
       </c>
-      <c r="D82" s="3" t="s">
+      <c r="E82" s="3" t="s">
         <v>486</v>
-      </c>
-      <c r="E82" s="3" t="s">
-        <v>487</v>
       </c>
       <c r="F82" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J82" s="3" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L82" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M82" s="1" t="s">
         <v>40</v>
@@ -6988,19 +6974,19 @@
         <v>118</v>
       </c>
       <c r="Z82" s="1" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="AA82" s="11" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="AB82" s="1" t="s">
-        <v>641</v>
+        <v>638</v>
       </c>
       <c r="AC82" s="1" t="s">
-        <v>659</v>
-      </c>
-    </row>
-    <row r="83" spans="1:29" ht="60" x14ac:dyDescent="0.25">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="83" spans="1:29" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" s="3">
         <v>82</v>
       </c>
@@ -7008,22 +6994,22 @@
         <v>24</v>
       </c>
       <c r="C83" s="3" t="s">
+        <v>489</v>
+      </c>
+      <c r="D83" s="3" t="s">
         <v>490</v>
       </c>
-      <c r="D83" s="3" t="s">
+      <c r="E83" s="3" t="s">
         <v>491</v>
-      </c>
-      <c r="E83" s="3" t="s">
-        <v>492</v>
       </c>
       <c r="F83" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J83" s="3" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L83" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M83" s="1" t="s">
         <v>40</v>
@@ -7045,13 +7031,13 @@
         <v>118</v>
       </c>
       <c r="AA83" s="11" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="AC83" s="1" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="84" spans="1:29" ht="60" x14ac:dyDescent="0.25">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="84" spans="1:29" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" s="3">
         <v>83</v>
       </c>
@@ -7059,22 +7045,22 @@
         <v>24</v>
       </c>
       <c r="C84" s="3" t="s">
+        <v>492</v>
+      </c>
+      <c r="D84" s="3" t="s">
         <v>493</v>
       </c>
-      <c r="D84" s="3" t="s">
+      <c r="E84" s="3" t="s">
         <v>494</v>
-      </c>
-      <c r="E84" s="3" t="s">
-        <v>495</v>
       </c>
       <c r="F84" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J84" s="3" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L84" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M84" s="1" t="s">
         <v>40</v>
@@ -7096,13 +7082,13 @@
         <v>118</v>
       </c>
       <c r="AA84" s="11" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="AC84" s="1" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="85" spans="1:29" ht="60" x14ac:dyDescent="0.25">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="85" spans="1:29" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="3">
         <v>84</v>
       </c>
@@ -7110,22 +7096,22 @@
         <v>24</v>
       </c>
       <c r="C85" s="3" t="s">
+        <v>495</v>
+      </c>
+      <c r="D85" s="3" t="s">
         <v>496</v>
       </c>
-      <c r="D85" s="3" t="s">
+      <c r="E85" s="3" t="s">
         <v>497</v>
-      </c>
-      <c r="E85" s="3" t="s">
-        <v>498</v>
       </c>
       <c r="F85" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J85" s="3" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L85" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M85" s="1" t="s">
         <v>40</v>
@@ -7147,13 +7133,13 @@
         <v>118</v>
       </c>
       <c r="AA85" s="11" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="AC85" s="1" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="86" spans="1:29" ht="60" x14ac:dyDescent="0.25">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="86" spans="1:29" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" s="3">
         <v>85</v>
       </c>
@@ -7161,22 +7147,22 @@
         <v>24</v>
       </c>
       <c r="C86" s="3" t="s">
+        <v>498</v>
+      </c>
+      <c r="D86" s="3" t="s">
         <v>499</v>
       </c>
-      <c r="D86" s="3" t="s">
+      <c r="E86" s="3" t="s">
         <v>500</v>
-      </c>
-      <c r="E86" s="3" t="s">
-        <v>501</v>
       </c>
       <c r="F86" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J86" s="3" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L86" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M86" s="1" t="s">
         <v>40</v>
@@ -7198,13 +7184,13 @@
         <v>118</v>
       </c>
       <c r="AA86" s="11" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="AC86" s="1" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="87" spans="1:29" ht="60" x14ac:dyDescent="0.25">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="87" spans="1:29" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" s="3">
         <v>86</v>
       </c>
@@ -7212,22 +7198,22 @@
         <v>24</v>
       </c>
       <c r="C87" s="3" t="s">
+        <v>501</v>
+      </c>
+      <c r="D87" s="3" t="s">
         <v>502</v>
       </c>
-      <c r="D87" s="3" t="s">
+      <c r="E87" s="3" t="s">
         <v>503</v>
-      </c>
-      <c r="E87" s="3" t="s">
-        <v>504</v>
       </c>
       <c r="F87" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J87" s="3" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L87" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M87" s="1" t="s">
         <v>40</v>
@@ -7249,13 +7235,13 @@
         <v>118</v>
       </c>
       <c r="AA87" s="11" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="AC87" s="1" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="88" spans="1:29" ht="60" x14ac:dyDescent="0.25">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="88" spans="1:29" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" s="3">
         <v>87</v>
       </c>
@@ -7263,22 +7249,22 @@
         <v>24</v>
       </c>
       <c r="C88" s="3" t="s">
+        <v>504</v>
+      </c>
+      <c r="D88" s="3" t="s">
         <v>505</v>
       </c>
-      <c r="D88" s="3" t="s">
+      <c r="E88" s="3" t="s">
         <v>506</v>
-      </c>
-      <c r="E88" s="3" t="s">
-        <v>507</v>
       </c>
       <c r="F88" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J88" s="3" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L88" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M88" s="1" t="s">
         <v>40</v>
@@ -7300,13 +7286,13 @@
         <v>118</v>
       </c>
       <c r="AA88" s="11" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="AC88" s="1" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="89" spans="1:29" ht="60" x14ac:dyDescent="0.25">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="89" spans="1:29" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" s="3">
         <v>88</v>
       </c>
@@ -7314,22 +7300,22 @@
         <v>24</v>
       </c>
       <c r="C89" s="3" t="s">
+        <v>507</v>
+      </c>
+      <c r="D89" s="3" t="s">
         <v>508</v>
       </c>
-      <c r="D89" s="3" t="s">
+      <c r="E89" s="3" t="s">
         <v>509</v>
-      </c>
-      <c r="E89" s="3" t="s">
-        <v>510</v>
       </c>
       <c r="F89" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J89" s="3" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L89" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M89" s="1" t="s">
         <v>40</v>
@@ -7351,13 +7337,13 @@
         <v>118</v>
       </c>
       <c r="AA89" s="11" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="AC89" s="1" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="90" spans="1:29" ht="60" x14ac:dyDescent="0.25">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="90" spans="1:29" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" s="3">
         <v>89</v>
       </c>
@@ -7365,22 +7351,22 @@
         <v>24</v>
       </c>
       <c r="C90" s="3" t="s">
+        <v>510</v>
+      </c>
+      <c r="D90" s="3" t="s">
         <v>511</v>
       </c>
-      <c r="D90" s="3" t="s">
+      <c r="E90" s="3" t="s">
         <v>512</v>
-      </c>
-      <c r="E90" s="3" t="s">
-        <v>513</v>
       </c>
       <c r="F90" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J90" s="3" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L90" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M90" s="1" t="s">
         <v>40</v>
@@ -7402,13 +7388,13 @@
         <v>118</v>
       </c>
       <c r="AA90" s="11" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="AC90" s="1" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="91" spans="1:29" ht="60" x14ac:dyDescent="0.25">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="91" spans="1:29" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" s="3">
         <v>90</v>
       </c>
@@ -7416,22 +7402,22 @@
         <v>24</v>
       </c>
       <c r="C91" s="3" t="s">
+        <v>513</v>
+      </c>
+      <c r="D91" s="3" t="s">
         <v>514</v>
       </c>
-      <c r="D91" s="3" t="s">
+      <c r="E91" s="3" t="s">
         <v>515</v>
-      </c>
-      <c r="E91" s="3" t="s">
-        <v>516</v>
       </c>
       <c r="F91" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J91" s="3" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L91" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M91" s="1" t="s">
         <v>40</v>
@@ -7453,13 +7439,13 @@
         <v>118</v>
       </c>
       <c r="AA91" s="11" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="AC91" s="1" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="92" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="92" spans="1:29" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" s="3">
         <v>91</v>
       </c>
@@ -7467,58 +7453,58 @@
         <v>24</v>
       </c>
       <c r="C92" s="3" t="s">
+        <v>516</v>
+      </c>
+      <c r="D92" s="3" t="s">
         <v>517</v>
       </c>
-      <c r="D92" s="3" t="s">
+      <c r="E92" s="3" t="s">
         <v>518</v>
-      </c>
-      <c r="E92" s="3" t="s">
-        <v>519</v>
       </c>
       <c r="F92" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J92" s="3" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L92" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M92" s="1" t="s">
         <v>40</v>
       </c>
       <c r="N92" s="1" t="s">
+        <v>519</v>
+      </c>
+      <c r="O92" s="9" t="s">
         <v>520</v>
       </c>
-      <c r="O92" s="9" t="s">
+      <c r="P92" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="V92" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="W92" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="X92" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="Y92" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="Z92" s="1" t="s">
         <v>521</v>
       </c>
-      <c r="P92" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="V92" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="W92" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="X92" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="Y92" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="Z92" s="1" t="s">
-        <v>522</v>
-      </c>
       <c r="AA92" s="11" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="AC92" s="3" t="s">
-        <v>657</v>
-      </c>
-    </row>
-    <row r="93" spans="1:29" ht="60" x14ac:dyDescent="0.25">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="93" spans="1:29" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" s="3">
         <v>92</v>
       </c>
@@ -7526,22 +7512,22 @@
         <v>24</v>
       </c>
       <c r="C93" s="3" t="s">
+        <v>522</v>
+      </c>
+      <c r="D93" s="3" t="s">
         <v>523</v>
       </c>
-      <c r="D93" s="3" t="s">
+      <c r="E93" s="3" t="s">
         <v>524</v>
-      </c>
-      <c r="E93" s="3" t="s">
-        <v>525</v>
       </c>
       <c r="F93" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J93" s="3" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L93" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M93" s="1" t="s">
         <v>40</v>
@@ -7563,13 +7549,13 @@
         <v>118</v>
       </c>
       <c r="AA93" s="11" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="AC93" s="1" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="94" spans="1:29" ht="60" x14ac:dyDescent="0.25">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="94" spans="1:29" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3">
         <v>93</v>
       </c>
@@ -7577,22 +7563,22 @@
         <v>24</v>
       </c>
       <c r="C94" s="3" t="s">
+        <v>525</v>
+      </c>
+      <c r="D94" s="3" t="s">
         <v>526</v>
       </c>
-      <c r="D94" s="3" t="s">
+      <c r="E94" s="3" t="s">
         <v>527</v>
-      </c>
-      <c r="E94" s="3" t="s">
-        <v>528</v>
       </c>
       <c r="F94" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J94" s="3" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L94" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M94" s="1" t="s">
         <v>40</v>
@@ -7614,13 +7600,13 @@
         <v>118</v>
       </c>
       <c r="AA94" s="11" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="AC94" s="1" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="95" spans="1:29" ht="60" x14ac:dyDescent="0.25">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="95" spans="1:29" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" s="3">
         <v>94</v>
       </c>
@@ -7628,22 +7614,22 @@
         <v>24</v>
       </c>
       <c r="C95" s="3" t="s">
+        <v>528</v>
+      </c>
+      <c r="D95" s="3" t="s">
         <v>529</v>
       </c>
-      <c r="D95" s="3" t="s">
+      <c r="E95" s="3" t="s">
         <v>530</v>
-      </c>
-      <c r="E95" s="3" t="s">
-        <v>531</v>
       </c>
       <c r="F95" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J95" s="3" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L95" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M95" s="1" t="s">
         <v>40</v>
@@ -7665,13 +7651,13 @@
         <v>118</v>
       </c>
       <c r="AA95" s="11" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="AC95" s="1" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="96" spans="1:29" ht="60" x14ac:dyDescent="0.25">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="96" spans="1:29" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" s="3">
         <v>95</v>
       </c>
@@ -7679,22 +7665,22 @@
         <v>24</v>
       </c>
       <c r="C96" s="3" t="s">
+        <v>531</v>
+      </c>
+      <c r="D96" s="3" t="s">
         <v>532</v>
       </c>
-      <c r="D96" s="3" t="s">
+      <c r="E96" s="3" t="s">
         <v>533</v>
-      </c>
-      <c r="E96" s="3" t="s">
-        <v>534</v>
       </c>
       <c r="F96" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J96" s="3" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L96" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M96" s="1" t="s">
         <v>40</v>
@@ -7716,13 +7702,13 @@
         <v>118</v>
       </c>
       <c r="AA96" s="11" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="AC96" s="1" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="97" spans="1:29" ht="60" x14ac:dyDescent="0.25">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="97" spans="1:29" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97" s="3">
         <v>96</v>
       </c>
@@ -7730,22 +7716,22 @@
         <v>24</v>
       </c>
       <c r="C97" s="3" t="s">
+        <v>534</v>
+      </c>
+      <c r="D97" s="3" t="s">
         <v>535</v>
       </c>
-      <c r="D97" s="3" t="s">
+      <c r="E97" s="3" t="s">
         <v>536</v>
-      </c>
-      <c r="E97" s="3" t="s">
-        <v>537</v>
       </c>
       <c r="F97" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J97" s="3" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L97" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M97" s="1" t="s">
         <v>40</v>
@@ -7767,13 +7753,13 @@
         <v>118</v>
       </c>
       <c r="AA97" s="11" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="AC97" s="1" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="98" spans="1:29" ht="60" x14ac:dyDescent="0.25">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="98" spans="1:29" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98" s="3">
         <v>97</v>
       </c>
@@ -7781,22 +7767,22 @@
         <v>24</v>
       </c>
       <c r="C98" s="3" t="s">
+        <v>537</v>
+      </c>
+      <c r="D98" s="3" t="s">
         <v>538</v>
       </c>
-      <c r="D98" s="3" t="s">
+      <c r="E98" s="3" t="s">
         <v>539</v>
-      </c>
-      <c r="E98" s="3" t="s">
-        <v>540</v>
       </c>
       <c r="F98" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J98" s="3" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L98" s="3" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M98" s="1" t="s">
         <v>40</v>
@@ -7818,13 +7804,13 @@
         <v>118</v>
       </c>
       <c r="AA98" s="11" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="AC98" s="1" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="99" spans="1:29" ht="60" x14ac:dyDescent="0.25">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="99" spans="1:29" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99" s="3">
         <v>98</v>
       </c>
@@ -7832,22 +7818,22 @@
         <v>24</v>
       </c>
       <c r="C99" s="3" t="s">
+        <v>540</v>
+      </c>
+      <c r="D99" s="3" t="s">
         <v>541</v>
       </c>
-      <c r="D99" s="3" t="s">
+      <c r="E99" s="3" t="s">
         <v>542</v>
-      </c>
-      <c r="E99" s="3" t="s">
-        <v>543</v>
       </c>
       <c r="F99" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J99" s="3" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L99" s="3" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M99" s="1" t="s">
         <v>40</v>
@@ -7869,13 +7855,13 @@
         <v>118</v>
       </c>
       <c r="AA99" s="11" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="AC99" s="1" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="100" spans="1:29" ht="60" x14ac:dyDescent="0.25">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="100" spans="1:29" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" s="3">
         <v>99</v>
       </c>
@@ -7883,22 +7869,22 @@
         <v>24</v>
       </c>
       <c r="C100" s="3" t="s">
+        <v>543</v>
+      </c>
+      <c r="D100" s="3" t="s">
         <v>544</v>
       </c>
-      <c r="D100" s="3" t="s">
+      <c r="E100" s="3" t="s">
         <v>545</v>
-      </c>
-      <c r="E100" s="3" t="s">
-        <v>546</v>
       </c>
       <c r="F100" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J100" s="3" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L100" s="3" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M100" s="1" t="s">
         <v>40</v>
@@ -7920,13 +7906,13 @@
         <v>118</v>
       </c>
       <c r="AA100" s="11" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="AC100" s="1" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="101" spans="1:29" x14ac:dyDescent="0.25">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="101" spans="1:29" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" s="3">
         <v>100</v>
       </c>
@@ -7934,22 +7920,22 @@
         <v>24</v>
       </c>
       <c r="C101" s="3" t="s">
+        <v>546</v>
+      </c>
+      <c r="D101" s="3" t="s">
         <v>547</v>
       </c>
-      <c r="D101" s="3" t="s">
+      <c r="E101" s="3" t="s">
         <v>548</v>
-      </c>
-      <c r="E101" s="3" t="s">
-        <v>549</v>
       </c>
       <c r="F101" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J101" s="3" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="L101" s="3" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M101" s="1" t="s">
         <v>40</v>
@@ -7971,7 +7957,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="102" spans="1:29" ht="90" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:29" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102" s="3">
         <v>101</v>
       </c>
@@ -7979,41 +7965,41 @@
         <v>24</v>
       </c>
       <c r="C102" s="3" t="s">
+        <v>550</v>
+      </c>
+      <c r="D102" s="3" t="s">
         <v>551</v>
       </c>
-      <c r="D102" s="3" t="s">
+      <c r="E102" s="3" t="s">
         <v>552</v>
-      </c>
-      <c r="E102" s="3" t="s">
-        <v>553</v>
       </c>
       <c r="F102" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J102" s="3" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="L102" s="3" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M102" s="11" t="s">
         <v>40</v>
       </c>
       <c r="N102" s="1" t="s">
-        <v>643</v>
+        <v>640</v>
       </c>
       <c r="O102" s="9"/>
       <c r="P102" s="3" t="s">
         <v>31</v>
       </c>
       <c r="T102" s="3" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
       <c r="V102" s="5" t="s">
         <v>88</v>
       </c>
       <c r="W102" s="5" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="X102" s="5" t="s">
         <v>88</v>
@@ -8022,13 +8008,13 @@
         <v>88</v>
       </c>
       <c r="Z102" s="1" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="AB102" s="11" t="s">
-        <v>642</v>
-      </c>
-    </row>
-    <row r="103" spans="1:29" x14ac:dyDescent="0.25">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="103" spans="1:29" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3">
         <v>102</v>
       </c>
@@ -8036,22 +8022,22 @@
         <v>24</v>
       </c>
       <c r="C103" s="3" t="s">
+        <v>555</v>
+      </c>
+      <c r="D103" s="3" t="s">
         <v>556</v>
       </c>
-      <c r="D103" s="3" t="s">
+      <c r="E103" s="3" t="s">
         <v>557</v>
-      </c>
-      <c r="E103" s="3" t="s">
-        <v>558</v>
       </c>
       <c r="F103" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J103" s="3" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="L103" s="3" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M103" s="1" t="s">
         <v>40</v>
@@ -8073,7 +8059,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="104" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:29" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104" s="3">
         <v>103</v>
       </c>
@@ -8081,31 +8067,31 @@
         <v>24</v>
       </c>
       <c r="C104" s="3" t="s">
+        <v>558</v>
+      </c>
+      <c r="D104" s="3" t="s">
         <v>559</v>
       </c>
-      <c r="D104" s="3" t="s">
-        <v>560</v>
-      </c>
       <c r="E104" s="3" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="F104" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J104" s="3" t="s">
+        <v>560</v>
+      </c>
+      <c r="L104" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="M104" s="1" t="s">
         <v>561</v>
       </c>
-      <c r="L104" s="3" t="s">
-        <v>404</v>
-      </c>
-      <c r="M104" s="1" t="s">
+      <c r="N104" s="3" t="s">
         <v>562</v>
       </c>
-      <c r="N104" s="3" t="s">
+      <c r="O104" s="1" t="s">
         <v>563</v>
-      </c>
-      <c r="O104" s="1" t="s">
-        <v>564</v>
       </c>
       <c r="P104" s="3" t="s">
         <v>31</v>
@@ -8123,10 +8109,10 @@
         <v>81</v>
       </c>
       <c r="Z104" s="1" t="s">
-        <v>565</v>
-      </c>
-    </row>
-    <row r="105" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="105" spans="1:29" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" s="3">
         <v>104</v>
       </c>
@@ -8134,31 +8120,31 @@
         <v>24</v>
       </c>
       <c r="C105" s="3" t="s">
+        <v>565</v>
+      </c>
+      <c r="D105" s="3" t="s">
         <v>566</v>
       </c>
-      <c r="D105" s="3" t="s">
-        <v>567</v>
-      </c>
       <c r="E105" s="3" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="F105" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J105" s="3" t="s">
+        <v>567</v>
+      </c>
+      <c r="L105" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="M105" s="1" t="s">
         <v>568</v>
       </c>
-      <c r="L105" s="3" t="s">
-        <v>404</v>
-      </c>
-      <c r="M105" s="1" t="s">
+      <c r="N105" s="3" t="s">
         <v>569</v>
       </c>
-      <c r="N105" s="3" t="s">
-        <v>570</v>
-      </c>
       <c r="O105" s="1" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="P105" s="3" t="s">
         <v>31</v>
@@ -8176,10 +8162,10 @@
         <v>81</v>
       </c>
       <c r="Z105" s="1" t="s">
-        <v>571</v>
-      </c>
-    </row>
-    <row r="106" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="106" spans="1:29" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106" s="3">
         <v>105</v>
       </c>
@@ -8187,31 +8173,31 @@
         <v>24</v>
       </c>
       <c r="C106" s="3" t="s">
+        <v>571</v>
+      </c>
+      <c r="D106" s="3" t="s">
         <v>572</v>
       </c>
-      <c r="D106" s="3" t="s">
-        <v>573</v>
-      </c>
       <c r="E106" s="3" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="F106" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J106" s="3" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="L106" s="3" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M106" s="1" t="s">
+        <v>573</v>
+      </c>
+      <c r="N106" s="1" t="s">
         <v>574</v>
       </c>
-      <c r="N106" s="1" t="s">
-        <v>575</v>
-      </c>
       <c r="O106" s="1" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="P106" s="3" t="s">
         <v>31</v>
@@ -8229,7 +8215,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="107" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:29" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107" s="3">
         <v>106</v>
       </c>
@@ -8237,19 +8223,19 @@
         <v>24</v>
       </c>
       <c r="C107" s="3" t="s">
+        <v>575</v>
+      </c>
+      <c r="D107" s="3" t="s">
         <v>576</v>
       </c>
-      <c r="D107" s="3" t="s">
-        <v>577</v>
-      </c>
       <c r="E107" s="3" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="F107" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J107" s="3" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="M107" s="1" t="s">
         <v>40</v>
@@ -8271,7 +8257,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="108" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:29" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108" s="3">
         <v>107</v>
       </c>
@@ -8279,19 +8265,19 @@
         <v>24</v>
       </c>
       <c r="C108" s="3" t="s">
+        <v>578</v>
+      </c>
+      <c r="D108" s="3" t="s">
         <v>579</v>
       </c>
-      <c r="D108" s="3" t="s">
-        <v>580</v>
-      </c>
       <c r="E108" s="3" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="F108" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J108" s="3" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="M108" s="1" t="s">
         <v>40</v>
@@ -8313,7 +8299,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="109" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:29" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109" s="3">
         <v>108</v>
       </c>
@@ -8321,19 +8307,19 @@
         <v>24</v>
       </c>
       <c r="C109" s="3" t="s">
+        <v>581</v>
+      </c>
+      <c r="D109" s="3" t="s">
         <v>582</v>
       </c>
-      <c r="D109" s="3" t="s">
-        <v>583</v>
-      </c>
       <c r="E109" s="3" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="F109" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J109" s="3" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="M109" s="1" t="s">
         <v>40</v>
@@ -8355,7 +8341,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="110" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:29" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110" s="3">
         <v>109</v>
       </c>
@@ -8363,19 +8349,19 @@
         <v>24</v>
       </c>
       <c r="C110" s="3" t="s">
+        <v>584</v>
+      </c>
+      <c r="D110" s="3" t="s">
         <v>585</v>
       </c>
-      <c r="D110" s="3" t="s">
-        <v>586</v>
-      </c>
       <c r="E110" s="3" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="F110" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J110" s="3" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="L110" s="1"/>
       <c r="M110" s="1" t="s">
@@ -8398,7 +8384,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="111" spans="1:29" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:29" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111" s="3">
         <v>110</v>
       </c>
@@ -8406,28 +8392,28 @@
         <v>24</v>
       </c>
       <c r="C111" s="3" t="s">
+        <v>587</v>
+      </c>
+      <c r="D111" s="3" t="s">
         <v>588</v>
       </c>
-      <c r="D111" s="3" t="s">
-        <v>589</v>
-      </c>
       <c r="E111" s="3" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="F111" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J111" s="3" t="s">
+        <v>589</v>
+      </c>
+      <c r="M111" s="1" t="s">
         <v>590</v>
       </c>
-      <c r="M111" s="1" t="s">
+      <c r="N111" s="1" t="s">
         <v>591</v>
       </c>
-      <c r="N111" s="1" t="s">
+      <c r="O111" s="1" t="s">
         <v>592</v>
-      </c>
-      <c r="O111" s="1" t="s">
-        <v>593</v>
       </c>
       <c r="P111" s="3" t="s">
         <v>31</v>
@@ -8442,13 +8428,13 @@
         <v>102</v>
       </c>
       <c r="Y111" s="10" t="s">
+        <v>593</v>
+      </c>
+      <c r="Z111" s="1" t="s">
         <v>594</v>
       </c>
-      <c r="Z111" s="1" t="s">
-        <v>595</v>
-      </c>
-    </row>
-    <row r="112" spans="1:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="112" spans="1:29" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112" s="3">
         <v>111</v>
       </c>
@@ -8456,19 +8442,19 @@
         <v>24</v>
       </c>
       <c r="C112" s="3" t="s">
+        <v>595</v>
+      </c>
+      <c r="D112" s="3" t="s">
         <v>596</v>
       </c>
-      <c r="D112" s="3" t="s">
-        <v>597</v>
-      </c>
       <c r="E112" s="3" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="F112" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J112" s="3" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="L112" s="1"/>
       <c r="M112" s="1" t="s">
@@ -8491,7 +8477,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="113" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113" s="3">
         <v>112</v>
       </c>
@@ -8499,19 +8485,19 @@
         <v>24</v>
       </c>
       <c r="C113" s="3" t="s">
+        <v>597</v>
+      </c>
+      <c r="D113" s="3" t="s">
         <v>598</v>
       </c>
-      <c r="D113" s="3" t="s">
-        <v>599</v>
-      </c>
       <c r="E113" s="3" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="F113" s="3" t="s">
         <v>50</v>
       </c>
       <c r="J113" s="3" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="L113" s="1"/>
       <c r="M113" s="1" t="s">
@@ -8535,7 +8521,54 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AF113" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:AF113" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="12">
+      <filters>
+        <filter val="activity_Q01_freq;_x000a_activity_Q02_frequency"/>
+        <filter val="activity_Q04_done ; _x000a_activity_Q09_done ; _x000a_activity_Q10_done ; _x000a_activity_Q11_done ; _x000a_activity_Q12_done ; _x000a_activity_Q14_done"/>
+        <filter val="Age.ph2"/>
+        <filter val="bmi.ph2"/>
+        <filter val="Deelnemer_ID"/>
+        <filter val="employ_cat.ph2"/>
+        <filter val="HbA1c_mol.ph2"/>
+        <filter val="HDL.ph2"/>
+        <filter val="Height.ph2"/>
+        <filter val="LDL.ph2"/>
+        <filter val="marital_status.ph2"/>
+        <filter val="med_DM.ph2"/>
+        <filter val="med_HT.ph2"/>
+        <filter val="med_LP.ph2"/>
+        <filter val="N_CVD.ph2"/>
+        <filter val="N_GTS_WHO.ph2"/>
+        <filter val="N_MajorGroup_ISCO08"/>
+        <filter val="nit_alcoholtot.ph2"/>
+        <filter val="nit_kcal.ph2"/>
+        <filter val="ODBP.ph2"/>
+        <filter val="OHR.ph2"/>
+        <filter val="OSBP.ph2"/>
+        <filter val="PHQ9_Q1.ph2 ; PHQ9_Q2.ph2 ;  PHQ9_Q3.ph2 ;  PHQ9_Q4.ph2 ;  PHQ9_Q5.ph2 ;  PHQ9_Q6.ph2 ;  PHQ9_Q7.ph2 ;  PHQ9_Q8.ph2 ;  PHQ9_Q9.ph2"/>
+        <filter val="PSQI_comp1_subjective_sleepquality"/>
+        <filter val="PSQI_comp3_sleep_duratation"/>
+        <filter val="SEX"/>
+        <filter val="SF36_Q01.ph2"/>
+        <filter val="SF36_Q03.ph2 ; SF36_Q04.ph2 ; SF36_Q05.ph2 ; SF36_Q06.ph2 ; SF36_Q07.ph2 ; SF36_Q08.ph2 ; SF36_Q09.ph2 ; SF36_Q10.ph2 ; SF36_Q11.ph2 ; SF36_Q12.ph2"/>
+        <filter val="smoking_4cat.ph2"/>
+        <filter val="Tot_chol.ph2"/>
+        <filter val="Tot_chol.ph2 ; HDL.ph2 ; Triglyc.ph2"/>
+        <filter val="TOTALPA.ph2"/>
+        <filter val="Triglyc.ph2"/>
+        <filter val="Visit1_date.ph2"/>
+        <filter val="waist.ph2"/>
+        <filter val="Weight.ph2"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="21">
+      <filters>
+        <filter val="impossible"/>
+        <filter val="undetermined"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200"/>
 </worksheet>

</xml_diff>